<commit_message>
added aug analysis; capacity limit
</commit_message>
<xml_diff>
--- a/4.0 FY2025 Material Control Fct 202507 (Jul - Mar).xlsx
+++ b/4.0 FY2025 Material Control Fct 202507 (Jul - Mar).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debdeeppaul/Documents/Procurement/PIDSG25/forecast25/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/debdeeppaul/Documents/Procurement/PIDSG25/pricesaa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D14C89CB-EA71-624A-9C28-2A2F7687AB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67364AFB-4215-9942-A850-616E3015B676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15760" xr2:uid="{5384D45F-16E8-4A35-B678-7039E9801426}"/>
   </bookViews>
@@ -1420,36 +1420,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="4" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="4" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1462,14 +1432,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="17" fontId="0" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="17" fontId="0" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="17" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1483,6 +1453,42 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="4" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="4" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1491,12 +1497,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2237,335 +2237,335 @@
       <c r="CL6" s="54"/>
     </row>
     <row r="7" spans="1:97" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="C7" s="172" t="s">
+      <c r="C7" s="169" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="175" t="s">
+      <c r="D7" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="176"/>
+      <c r="E7" s="166"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="165">
+      <c r="G7" s="162">
         <v>45748</v>
       </c>
-      <c r="H7" s="166"/>
-      <c r="I7" s="166"/>
-      <c r="J7" s="166"/>
-      <c r="K7" s="166"/>
-      <c r="L7" s="166"/>
-      <c r="M7" s="167"/>
-      <c r="N7" s="165">
+      <c r="H7" s="163"/>
+      <c r="I7" s="163"/>
+      <c r="J7" s="163"/>
+      <c r="K7" s="163"/>
+      <c r="L7" s="163"/>
+      <c r="M7" s="164"/>
+      <c r="N7" s="162">
         <v>45778</v>
       </c>
-      <c r="O7" s="166"/>
-      <c r="P7" s="166"/>
-      <c r="Q7" s="166"/>
-      <c r="R7" s="166"/>
-      <c r="S7" s="166"/>
-      <c r="T7" s="167"/>
-      <c r="U7" s="165">
+      <c r="O7" s="163"/>
+      <c r="P7" s="163"/>
+      <c r="Q7" s="163"/>
+      <c r="R7" s="163"/>
+      <c r="S7" s="163"/>
+      <c r="T7" s="164"/>
+      <c r="U7" s="162">
         <v>45809</v>
       </c>
-      <c r="V7" s="166"/>
-      <c r="W7" s="166"/>
-      <c r="X7" s="166"/>
-      <c r="Y7" s="166"/>
-      <c r="Z7" s="166"/>
-      <c r="AA7" s="167"/>
-      <c r="AB7" s="165">
+      <c r="V7" s="163"/>
+      <c r="W7" s="163"/>
+      <c r="X7" s="163"/>
+      <c r="Y7" s="163"/>
+      <c r="Z7" s="163"/>
+      <c r="AA7" s="164"/>
+      <c r="AB7" s="162">
         <v>45839</v>
       </c>
-      <c r="AC7" s="166"/>
-      <c r="AD7" s="166"/>
-      <c r="AE7" s="166"/>
-      <c r="AF7" s="166"/>
-      <c r="AG7" s="166"/>
-      <c r="AH7" s="167"/>
-      <c r="AI7" s="165">
+      <c r="AC7" s="163"/>
+      <c r="AD7" s="163"/>
+      <c r="AE7" s="163"/>
+      <c r="AF7" s="163"/>
+      <c r="AG7" s="163"/>
+      <c r="AH7" s="164"/>
+      <c r="AI7" s="162">
         <v>45870</v>
       </c>
-      <c r="AJ7" s="166"/>
-      <c r="AK7" s="166"/>
-      <c r="AL7" s="166"/>
-      <c r="AM7" s="166"/>
-      <c r="AN7" s="166"/>
-      <c r="AO7" s="167"/>
-      <c r="AP7" s="165">
+      <c r="AJ7" s="163"/>
+      <c r="AK7" s="163"/>
+      <c r="AL7" s="163"/>
+      <c r="AM7" s="163"/>
+      <c r="AN7" s="163"/>
+      <c r="AO7" s="164"/>
+      <c r="AP7" s="162">
         <v>45901</v>
       </c>
-      <c r="AQ7" s="166"/>
-      <c r="AR7" s="166"/>
-      <c r="AS7" s="166"/>
-      <c r="AT7" s="166"/>
-      <c r="AU7" s="166"/>
-      <c r="AV7" s="167"/>
-      <c r="AW7" s="165">
+      <c r="AQ7" s="163"/>
+      <c r="AR7" s="163"/>
+      <c r="AS7" s="163"/>
+      <c r="AT7" s="163"/>
+      <c r="AU7" s="163"/>
+      <c r="AV7" s="164"/>
+      <c r="AW7" s="162">
         <v>45931</v>
       </c>
-      <c r="AX7" s="166"/>
-      <c r="AY7" s="166"/>
-      <c r="AZ7" s="166"/>
-      <c r="BA7" s="166"/>
-      <c r="BB7" s="166"/>
-      <c r="BC7" s="167"/>
-      <c r="BD7" s="165">
+      <c r="AX7" s="163"/>
+      <c r="AY7" s="163"/>
+      <c r="AZ7" s="163"/>
+      <c r="BA7" s="163"/>
+      <c r="BB7" s="163"/>
+      <c r="BC7" s="164"/>
+      <c r="BD7" s="162">
         <v>45962</v>
       </c>
-      <c r="BE7" s="166"/>
-      <c r="BF7" s="166"/>
-      <c r="BG7" s="166"/>
-      <c r="BH7" s="166"/>
-      <c r="BI7" s="166"/>
-      <c r="BJ7" s="167"/>
-      <c r="BK7" s="165">
+      <c r="BE7" s="163"/>
+      <c r="BF7" s="163"/>
+      <c r="BG7" s="163"/>
+      <c r="BH7" s="163"/>
+      <c r="BI7" s="163"/>
+      <c r="BJ7" s="164"/>
+      <c r="BK7" s="162">
         <v>45992</v>
       </c>
-      <c r="BL7" s="166"/>
-      <c r="BM7" s="166"/>
-      <c r="BN7" s="166"/>
-      <c r="BO7" s="166"/>
-      <c r="BP7" s="166"/>
-      <c r="BQ7" s="167"/>
-      <c r="BR7" s="165">
+      <c r="BL7" s="163"/>
+      <c r="BM7" s="163"/>
+      <c r="BN7" s="163"/>
+      <c r="BO7" s="163"/>
+      <c r="BP7" s="163"/>
+      <c r="BQ7" s="164"/>
+      <c r="BR7" s="162">
         <v>46023</v>
       </c>
-      <c r="BS7" s="166"/>
-      <c r="BT7" s="166"/>
-      <c r="BU7" s="166"/>
-      <c r="BV7" s="166"/>
-      <c r="BW7" s="166"/>
-      <c r="BX7" s="167"/>
-      <c r="BY7" s="165">
+      <c r="BS7" s="163"/>
+      <c r="BT7" s="163"/>
+      <c r="BU7" s="163"/>
+      <c r="BV7" s="163"/>
+      <c r="BW7" s="163"/>
+      <c r="BX7" s="164"/>
+      <c r="BY7" s="162">
         <v>46054</v>
       </c>
-      <c r="BZ7" s="166"/>
-      <c r="CA7" s="166"/>
-      <c r="CB7" s="166"/>
-      <c r="CC7" s="166"/>
-      <c r="CD7" s="166"/>
-      <c r="CE7" s="167"/>
-      <c r="CF7" s="165">
+      <c r="BZ7" s="163"/>
+      <c r="CA7" s="163"/>
+      <c r="CB7" s="163"/>
+      <c r="CC7" s="163"/>
+      <c r="CD7" s="163"/>
+      <c r="CE7" s="164"/>
+      <c r="CF7" s="162">
         <v>46082</v>
       </c>
-      <c r="CG7" s="166"/>
-      <c r="CH7" s="166"/>
-      <c r="CI7" s="166"/>
-      <c r="CJ7" s="166"/>
-      <c r="CK7" s="166"/>
-      <c r="CL7" s="167"/>
-      <c r="CM7" s="165" t="s">
+      <c r="CG7" s="163"/>
+      <c r="CH7" s="163"/>
+      <c r="CI7" s="163"/>
+      <c r="CJ7" s="163"/>
+      <c r="CK7" s="163"/>
+      <c r="CL7" s="164"/>
+      <c r="CM7" s="162" t="s">
         <v>3</v>
       </c>
-      <c r="CN7" s="166"/>
-      <c r="CO7" s="166"/>
-      <c r="CP7" s="166"/>
-      <c r="CQ7" s="166"/>
-      <c r="CR7" s="166"/>
-      <c r="CS7" s="167"/>
+      <c r="CN7" s="163"/>
+      <c r="CO7" s="163"/>
+      <c r="CP7" s="163"/>
+      <c r="CQ7" s="163"/>
+      <c r="CR7" s="163"/>
+      <c r="CS7" s="164"/>
     </row>
     <row r="8" spans="1:97" x14ac:dyDescent="0.2">
-      <c r="C8" s="173"/>
-      <c r="D8" s="182" t="s">
+      <c r="C8" s="170"/>
+      <c r="D8" s="172" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="177" t="s">
+      <c r="E8" s="167" t="s">
         <v>5</v>
       </c>
       <c r="F8" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="168" t="s">
+      <c r="G8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="H8" s="169"/>
-      <c r="I8" s="170" t="s">
+      <c r="H8" s="159"/>
+      <c r="I8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="J8" s="169"/>
-      <c r="K8" s="170" t="s">
+      <c r="J8" s="159"/>
+      <c r="K8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="L8" s="171"/>
+      <c r="L8" s="161"/>
       <c r="M8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="N8" s="168" t="s">
+      <c r="N8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="O8" s="169"/>
-      <c r="P8" s="170" t="s">
+      <c r="O8" s="159"/>
+      <c r="P8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="Q8" s="169"/>
-      <c r="R8" s="170" t="s">
+      <c r="Q8" s="159"/>
+      <c r="R8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="S8" s="171"/>
+      <c r="S8" s="161"/>
       <c r="T8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="U8" s="168" t="s">
+      <c r="U8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="V8" s="169"/>
-      <c r="W8" s="170" t="s">
+      <c r="V8" s="159"/>
+      <c r="W8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="X8" s="169"/>
-      <c r="Y8" s="170" t="s">
+      <c r="X8" s="159"/>
+      <c r="Y8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="Z8" s="171"/>
+      <c r="Z8" s="161"/>
       <c r="AA8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="AB8" s="168" t="s">
+      <c r="AB8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="AC8" s="169"/>
-      <c r="AD8" s="170" t="s">
+      <c r="AC8" s="159"/>
+      <c r="AD8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="AE8" s="169"/>
-      <c r="AF8" s="170" t="s">
+      <c r="AE8" s="159"/>
+      <c r="AF8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="AG8" s="171"/>
+      <c r="AG8" s="161"/>
       <c r="AH8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="AI8" s="171" t="s">
+      <c r="AI8" s="161" t="s">
         <v>7</v>
       </c>
-      <c r="AJ8" s="169"/>
-      <c r="AK8" s="170" t="s">
+      <c r="AJ8" s="159"/>
+      <c r="AK8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="AL8" s="169"/>
-      <c r="AM8" s="170" t="s">
+      <c r="AL8" s="159"/>
+      <c r="AM8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="AN8" s="171"/>
+      <c r="AN8" s="161"/>
       <c r="AO8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="AP8" s="168" t="s">
+      <c r="AP8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="AQ8" s="169"/>
-      <c r="AR8" s="170" t="s">
+      <c r="AQ8" s="159"/>
+      <c r="AR8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="AS8" s="169"/>
-      <c r="AT8" s="170" t="s">
+      <c r="AS8" s="159"/>
+      <c r="AT8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="AU8" s="171"/>
+      <c r="AU8" s="161"/>
       <c r="AV8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="AW8" s="168" t="s">
+      <c r="AW8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="AX8" s="169"/>
-      <c r="AY8" s="170" t="s">
+      <c r="AX8" s="159"/>
+      <c r="AY8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="AZ8" s="169"/>
-      <c r="BA8" s="170" t="s">
+      <c r="AZ8" s="159"/>
+      <c r="BA8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="BB8" s="171"/>
+      <c r="BB8" s="161"/>
       <c r="BC8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="BD8" s="168" t="s">
+      <c r="BD8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="BE8" s="169"/>
-      <c r="BF8" s="170" t="s">
+      <c r="BE8" s="159"/>
+      <c r="BF8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="BG8" s="169"/>
-      <c r="BH8" s="170" t="s">
+      <c r="BG8" s="159"/>
+      <c r="BH8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="BI8" s="171"/>
+      <c r="BI8" s="161"/>
       <c r="BJ8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="BK8" s="168" t="s">
+      <c r="BK8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="BL8" s="169"/>
-      <c r="BM8" s="170" t="s">
+      <c r="BL8" s="159"/>
+      <c r="BM8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="BN8" s="169"/>
-      <c r="BO8" s="170" t="s">
+      <c r="BN8" s="159"/>
+      <c r="BO8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="BP8" s="171"/>
+      <c r="BP8" s="161"/>
       <c r="BQ8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="BR8" s="168" t="s">
+      <c r="BR8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="BS8" s="169"/>
-      <c r="BT8" s="170" t="s">
+      <c r="BS8" s="159"/>
+      <c r="BT8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="BU8" s="169"/>
-      <c r="BV8" s="170" t="s">
+      <c r="BU8" s="159"/>
+      <c r="BV8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="BW8" s="171"/>
+      <c r="BW8" s="161"/>
       <c r="BX8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="BY8" s="168" t="s">
+      <c r="BY8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="BZ8" s="169"/>
-      <c r="CA8" s="170" t="s">
+      <c r="BZ8" s="159"/>
+      <c r="CA8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="CB8" s="169"/>
-      <c r="CC8" s="170" t="s">
+      <c r="CB8" s="159"/>
+      <c r="CC8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="CD8" s="171"/>
+      <c r="CD8" s="161"/>
       <c r="CE8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="CF8" s="168" t="s">
+      <c r="CF8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="CG8" s="169"/>
-      <c r="CH8" s="170" t="s">
+      <c r="CG8" s="159"/>
+      <c r="CH8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="CI8" s="169"/>
-      <c r="CJ8" s="170" t="s">
+      <c r="CI8" s="159"/>
+      <c r="CJ8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="CK8" s="171"/>
+      <c r="CK8" s="161"/>
       <c r="CL8" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="CM8" s="168" t="s">
+      <c r="CM8" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="CN8" s="169"/>
-      <c r="CO8" s="170" t="s">
+      <c r="CN8" s="159"/>
+      <c r="CO8" s="160" t="s">
         <v>8</v>
       </c>
-      <c r="CP8" s="169"/>
-      <c r="CQ8" s="170" t="s">
+      <c r="CP8" s="159"/>
+      <c r="CQ8" s="160" t="s">
         <v>6</v>
       </c>
-      <c r="CR8" s="171"/>
+      <c r="CR8" s="161"/>
       <c r="CS8" s="66" t="s">
         <v>9</v>
       </c>
@@ -2573,9 +2573,9 @@
     <row r="9" spans="1:97" ht="17.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="67"/>
       <c r="B9" s="67"/>
-      <c r="C9" s="174"/>
-      <c r="D9" s="183"/>
-      <c r="E9" s="178"/>
+      <c r="C9" s="171"/>
+      <c r="D9" s="173"/>
+      <c r="E9" s="168"/>
       <c r="F9" s="39" t="s">
         <v>10</v>
       </c>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="CS19" s="101"/>
     </row>
-    <row r="20" spans="1:111" s="123" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:111" s="123" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C20" s="124"/>
       <c r="D20" s="71"/>
       <c r="E20" s="125"/>
@@ -5694,7 +5694,7 @@
       <c r="CL20" s="71"/>
       <c r="CM20" s="97"/>
     </row>
-    <row r="21" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:111" x14ac:dyDescent="0.2">
       <c r="G21" s="70"/>
       <c r="H21" s="70"/>
       <c r="I21" s="70"/>
@@ -5785,7 +5785,7 @@
       <c r="CQ21" s="70"/>
       <c r="CR21" s="70"/>
     </row>
-    <row r="22" spans="1:111" ht="18.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:111" ht="18.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C22" s="88"/>
       <c r="H22" s="54"/>
       <c r="I22" s="54"/>
@@ -5869,409 +5869,409 @@
       </c>
       <c r="CL22" s="54"/>
     </row>
-    <row r="23" spans="1:111" ht="15" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="C23" s="172" t="s">
+    <row r="23" spans="1:111" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="C23" s="169" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="175" t="s">
+      <c r="D23" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="E23" s="176"/>
+      <c r="E23" s="166"/>
       <c r="F23" s="1"/>
-      <c r="G23" s="165">
+      <c r="G23" s="162">
         <f>G$7</f>
         <v>45748</v>
       </c>
-      <c r="H23" s="166"/>
-      <c r="I23" s="166"/>
-      <c r="J23" s="166"/>
-      <c r="K23" s="166"/>
-      <c r="L23" s="166"/>
-      <c r="M23" s="167"/>
-      <c r="N23" s="165">
+      <c r="H23" s="163"/>
+      <c r="I23" s="163"/>
+      <c r="J23" s="163"/>
+      <c r="K23" s="163"/>
+      <c r="L23" s="163"/>
+      <c r="M23" s="164"/>
+      <c r="N23" s="162">
         <f>N$7</f>
         <v>45778</v>
       </c>
-      <c r="O23" s="166"/>
-      <c r="P23" s="166"/>
-      <c r="Q23" s="166"/>
-      <c r="R23" s="166"/>
-      <c r="S23" s="166"/>
-      <c r="T23" s="167"/>
-      <c r="U23" s="165">
+      <c r="O23" s="163"/>
+      <c r="P23" s="163"/>
+      <c r="Q23" s="163"/>
+      <c r="R23" s="163"/>
+      <c r="S23" s="163"/>
+      <c r="T23" s="164"/>
+      <c r="U23" s="162">
         <f>U$7</f>
         <v>45809</v>
       </c>
-      <c r="V23" s="166"/>
-      <c r="W23" s="166"/>
-      <c r="X23" s="166"/>
-      <c r="Y23" s="166"/>
-      <c r="Z23" s="166"/>
-      <c r="AA23" s="167"/>
-      <c r="AB23" s="165">
+      <c r="V23" s="163"/>
+      <c r="W23" s="163"/>
+      <c r="X23" s="163"/>
+      <c r="Y23" s="163"/>
+      <c r="Z23" s="163"/>
+      <c r="AA23" s="164"/>
+      <c r="AB23" s="162">
         <f>AB$7</f>
         <v>45839</v>
       </c>
-      <c r="AC23" s="166"/>
-      <c r="AD23" s="166"/>
-      <c r="AE23" s="166"/>
-      <c r="AF23" s="166"/>
-      <c r="AG23" s="166"/>
-      <c r="AH23" s="167"/>
-      <c r="AI23" s="165">
+      <c r="AC23" s="163"/>
+      <c r="AD23" s="163"/>
+      <c r="AE23" s="163"/>
+      <c r="AF23" s="163"/>
+      <c r="AG23" s="163"/>
+      <c r="AH23" s="164"/>
+      <c r="AI23" s="162">
         <f>AI$7</f>
         <v>45870</v>
       </c>
-      <c r="AJ23" s="166"/>
-      <c r="AK23" s="166"/>
-      <c r="AL23" s="166"/>
-      <c r="AM23" s="166"/>
-      <c r="AN23" s="166"/>
-      <c r="AO23" s="167"/>
-      <c r="AP23" s="165">
+      <c r="AJ23" s="163"/>
+      <c r="AK23" s="163"/>
+      <c r="AL23" s="163"/>
+      <c r="AM23" s="163"/>
+      <c r="AN23" s="163"/>
+      <c r="AO23" s="164"/>
+      <c r="AP23" s="162">
         <f>AP$7</f>
         <v>45901</v>
       </c>
-      <c r="AQ23" s="166"/>
-      <c r="AR23" s="166"/>
-      <c r="AS23" s="166"/>
-      <c r="AT23" s="166"/>
-      <c r="AU23" s="166"/>
-      <c r="AV23" s="167"/>
-      <c r="AW23" s="165">
+      <c r="AQ23" s="163"/>
+      <c r="AR23" s="163"/>
+      <c r="AS23" s="163"/>
+      <c r="AT23" s="163"/>
+      <c r="AU23" s="163"/>
+      <c r="AV23" s="164"/>
+      <c r="AW23" s="162">
         <f>AW$7</f>
         <v>45931</v>
       </c>
-      <c r="AX23" s="166"/>
-      <c r="AY23" s="166"/>
-      <c r="AZ23" s="166"/>
-      <c r="BA23" s="166"/>
-      <c r="BB23" s="166"/>
-      <c r="BC23" s="167"/>
-      <c r="BD23" s="165">
+      <c r="AX23" s="163"/>
+      <c r="AY23" s="163"/>
+      <c r="AZ23" s="163"/>
+      <c r="BA23" s="163"/>
+      <c r="BB23" s="163"/>
+      <c r="BC23" s="164"/>
+      <c r="BD23" s="162">
         <f>BD$7</f>
         <v>45962</v>
       </c>
-      <c r="BE23" s="166"/>
-      <c r="BF23" s="166"/>
-      <c r="BG23" s="166"/>
-      <c r="BH23" s="166"/>
-      <c r="BI23" s="166"/>
-      <c r="BJ23" s="167"/>
-      <c r="BK23" s="165">
+      <c r="BE23" s="163"/>
+      <c r="BF23" s="163"/>
+      <c r="BG23" s="163"/>
+      <c r="BH23" s="163"/>
+      <c r="BI23" s="163"/>
+      <c r="BJ23" s="164"/>
+      <c r="BK23" s="162">
         <f>BK$7</f>
         <v>45992</v>
       </c>
-      <c r="BL23" s="166"/>
-      <c r="BM23" s="166"/>
-      <c r="BN23" s="166"/>
-      <c r="BO23" s="166"/>
-      <c r="BP23" s="166"/>
-      <c r="BQ23" s="167"/>
-      <c r="BR23" s="165">
+      <c r="BL23" s="163"/>
+      <c r="BM23" s="163"/>
+      <c r="BN23" s="163"/>
+      <c r="BO23" s="163"/>
+      <c r="BP23" s="163"/>
+      <c r="BQ23" s="164"/>
+      <c r="BR23" s="162">
         <f>BR$7</f>
         <v>46023</v>
       </c>
-      <c r="BS23" s="166"/>
-      <c r="BT23" s="166"/>
-      <c r="BU23" s="166"/>
-      <c r="BV23" s="166"/>
-      <c r="BW23" s="166"/>
-      <c r="BX23" s="167"/>
-      <c r="BY23" s="165">
+      <c r="BS23" s="163"/>
+      <c r="BT23" s="163"/>
+      <c r="BU23" s="163"/>
+      <c r="BV23" s="163"/>
+      <c r="BW23" s="163"/>
+      <c r="BX23" s="164"/>
+      <c r="BY23" s="162">
         <f>BY$7</f>
         <v>46054</v>
       </c>
-      <c r="BZ23" s="166"/>
-      <c r="CA23" s="166"/>
-      <c r="CB23" s="166"/>
-      <c r="CC23" s="166"/>
-      <c r="CD23" s="166"/>
-      <c r="CE23" s="167"/>
-      <c r="CF23" s="165">
+      <c r="BZ23" s="163"/>
+      <c r="CA23" s="163"/>
+      <c r="CB23" s="163"/>
+      <c r="CC23" s="163"/>
+      <c r="CD23" s="163"/>
+      <c r="CE23" s="164"/>
+      <c r="CF23" s="162">
         <f>CF$7</f>
         <v>46082</v>
       </c>
-      <c r="CG23" s="166"/>
-      <c r="CH23" s="166"/>
-      <c r="CI23" s="166"/>
-      <c r="CJ23" s="166"/>
-      <c r="CK23" s="166"/>
-      <c r="CL23" s="167"/>
-      <c r="CM23" s="165" t="str">
+      <c r="CG23" s="163"/>
+      <c r="CH23" s="163"/>
+      <c r="CI23" s="163"/>
+      <c r="CJ23" s="163"/>
+      <c r="CK23" s="163"/>
+      <c r="CL23" s="164"/>
+      <c r="CM23" s="162" t="str">
         <f t="shared" ref="CM23" si="65">CM$7</f>
         <v>FY26 1H</v>
       </c>
-      <c r="CN23" s="166"/>
-      <c r="CO23" s="166"/>
-      <c r="CP23" s="166"/>
-      <c r="CQ23" s="166"/>
-      <c r="CR23" s="166"/>
-      <c r="CS23" s="167"/>
+      <c r="CN23" s="163"/>
+      <c r="CO23" s="163"/>
+      <c r="CP23" s="163"/>
+      <c r="CQ23" s="163"/>
+      <c r="CR23" s="163"/>
+      <c r="CS23" s="164"/>
     </row>
-    <row r="24" spans="1:111" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C24" s="173"/>
-      <c r="D24" s="182" t="s">
+    <row r="24" spans="1:111" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C24" s="170"/>
+      <c r="D24" s="172" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="177" t="s">
+      <c r="E24" s="167" t="s">
         <v>5</v>
       </c>
       <c r="F24" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="G24" s="168" t="str">
+      <c r="G24" s="158" t="str">
         <f>G$8</f>
         <v>Pur</v>
       </c>
-      <c r="H24" s="169"/>
-      <c r="I24" s="170" t="str">
+      <c r="H24" s="159"/>
+      <c r="I24" s="160" t="str">
         <f>I$8</f>
         <v>Consumption</v>
       </c>
-      <c r="J24" s="169"/>
-      <c r="K24" s="170" t="str">
+      <c r="J24" s="159"/>
+      <c r="K24" s="160" t="str">
         <f>K$8</f>
         <v>C/B</v>
       </c>
-      <c r="L24" s="171"/>
+      <c r="L24" s="161"/>
       <c r="M24" s="66" t="str">
         <f>M$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="N24" s="168" t="str">
+      <c r="N24" s="158" t="str">
         <f>N$8</f>
         <v>Pur</v>
       </c>
-      <c r="O24" s="169"/>
-      <c r="P24" s="170" t="str">
+      <c r="O24" s="159"/>
+      <c r="P24" s="160" t="str">
         <f>P$8</f>
         <v>Consumption</v>
       </c>
-      <c r="Q24" s="169"/>
-      <c r="R24" s="170" t="str">
+      <c r="Q24" s="159"/>
+      <c r="R24" s="160" t="str">
         <f>R$8</f>
         <v>C/B</v>
       </c>
-      <c r="S24" s="171"/>
+      <c r="S24" s="161"/>
       <c r="T24" s="66" t="str">
         <f t="shared" ref="T24" si="66">T$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="U24" s="168" t="str">
+      <c r="U24" s="158" t="str">
         <f t="shared" ref="U24" si="67">U$8</f>
         <v>Pur</v>
       </c>
-      <c r="V24" s="169"/>
-      <c r="W24" s="170" t="str">
+      <c r="V24" s="159"/>
+      <c r="W24" s="160" t="str">
         <f t="shared" ref="W24" si="68">W$8</f>
         <v>Consumption</v>
       </c>
-      <c r="X24" s="169"/>
-      <c r="Y24" s="170" t="str">
+      <c r="X24" s="159"/>
+      <c r="Y24" s="160" t="str">
         <f t="shared" ref="Y24" si="69">Y$8</f>
         <v>C/B</v>
       </c>
-      <c r="Z24" s="171"/>
+      <c r="Z24" s="161"/>
       <c r="AA24" s="66" t="str">
         <f t="shared" ref="AA24:AB24" si="70">AA$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AB24" s="168" t="str">
+      <c r="AB24" s="158" t="str">
         <f t="shared" si="70"/>
         <v>Pur</v>
       </c>
-      <c r="AC24" s="169"/>
-      <c r="AD24" s="170" t="str">
+      <c r="AC24" s="159"/>
+      <c r="AD24" s="160" t="str">
         <f t="shared" ref="AD24" si="71">AD$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AE24" s="169"/>
-      <c r="AF24" s="170" t="str">
+      <c r="AE24" s="159"/>
+      <c r="AF24" s="160" t="str">
         <f t="shared" ref="AF24" si="72">AF$8</f>
         <v>C/B</v>
       </c>
-      <c r="AG24" s="171"/>
+      <c r="AG24" s="161"/>
       <c r="AH24" s="66" t="str">
         <f t="shared" ref="AH24:AI24" si="73">AH$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AI24" s="168" t="str">
+      <c r="AI24" s="158" t="str">
         <f t="shared" si="73"/>
         <v>Pur</v>
       </c>
-      <c r="AJ24" s="169"/>
-      <c r="AK24" s="170" t="str">
+      <c r="AJ24" s="159"/>
+      <c r="AK24" s="160" t="str">
         <f t="shared" ref="AK24" si="74">AK$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AL24" s="169"/>
-      <c r="AM24" s="170" t="str">
+      <c r="AL24" s="159"/>
+      <c r="AM24" s="160" t="str">
         <f t="shared" ref="AM24" si="75">AM$8</f>
         <v>C/B</v>
       </c>
-      <c r="AN24" s="171"/>
+      <c r="AN24" s="161"/>
       <c r="AO24" s="66" t="str">
         <f t="shared" ref="AO24:AP24" si="76">AO$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AP24" s="168" t="str">
+      <c r="AP24" s="158" t="str">
         <f t="shared" si="76"/>
         <v>Pur</v>
       </c>
-      <c r="AQ24" s="169"/>
-      <c r="AR24" s="170" t="str">
+      <c r="AQ24" s="159"/>
+      <c r="AR24" s="160" t="str">
         <f t="shared" ref="AR24" si="77">AR$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AS24" s="169"/>
-      <c r="AT24" s="170" t="str">
+      <c r="AS24" s="159"/>
+      <c r="AT24" s="160" t="str">
         <f t="shared" ref="AT24" si="78">AT$8</f>
         <v>C/B</v>
       </c>
-      <c r="AU24" s="171"/>
+      <c r="AU24" s="161"/>
       <c r="AV24" s="66" t="str">
         <f t="shared" ref="AV24" si="79">AV$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AW24" s="168" t="str">
+      <c r="AW24" s="158" t="str">
         <f t="shared" ref="AW24" si="80">AW$8</f>
         <v>Pur</v>
       </c>
-      <c r="AX24" s="169"/>
-      <c r="AY24" s="170" t="str">
+      <c r="AX24" s="159"/>
+      <c r="AY24" s="160" t="str">
         <f t="shared" ref="AY24" si="81">AY$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AZ24" s="169"/>
-      <c r="BA24" s="170" t="str">
+      <c r="AZ24" s="159"/>
+      <c r="BA24" s="160" t="str">
         <f t="shared" ref="BA24" si="82">BA$8</f>
         <v>C/B</v>
       </c>
-      <c r="BB24" s="171"/>
+      <c r="BB24" s="161"/>
       <c r="BC24" s="66" t="str">
         <f t="shared" ref="BC24:BD24" si="83">BC$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BD24" s="168" t="str">
+      <c r="BD24" s="158" t="str">
         <f t="shared" si="83"/>
         <v>Pur</v>
       </c>
-      <c r="BE24" s="169"/>
-      <c r="BF24" s="170" t="str">
+      <c r="BE24" s="159"/>
+      <c r="BF24" s="160" t="str">
         <f t="shared" ref="BF24" si="84">BF$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BG24" s="169"/>
-      <c r="BH24" s="170" t="str">
+      <c r="BG24" s="159"/>
+      <c r="BH24" s="160" t="str">
         <f t="shared" ref="BH24" si="85">BH$8</f>
         <v>C/B</v>
       </c>
-      <c r="BI24" s="171"/>
+      <c r="BI24" s="161"/>
       <c r="BJ24" s="66" t="str">
         <f t="shared" ref="BJ24:BK24" si="86">BJ$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BK24" s="168" t="str">
+      <c r="BK24" s="158" t="str">
         <f t="shared" si="86"/>
         <v>Pur</v>
       </c>
-      <c r="BL24" s="169"/>
-      <c r="BM24" s="170" t="str">
+      <c r="BL24" s="159"/>
+      <c r="BM24" s="160" t="str">
         <f t="shared" ref="BM24" si="87">BM$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BN24" s="169"/>
-      <c r="BO24" s="170" t="str">
+      <c r="BN24" s="159"/>
+      <c r="BO24" s="160" t="str">
         <f t="shared" ref="BO24" si="88">BO$8</f>
         <v>C/B</v>
       </c>
-      <c r="BP24" s="171"/>
+      <c r="BP24" s="161"/>
       <c r="BQ24" s="66" t="str">
         <f t="shared" ref="BQ24:BR24" si="89">BQ$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BR24" s="168" t="str">
+      <c r="BR24" s="158" t="str">
         <f t="shared" si="89"/>
         <v>Pur</v>
       </c>
-      <c r="BS24" s="169"/>
-      <c r="BT24" s="170" t="str">
+      <c r="BS24" s="159"/>
+      <c r="BT24" s="160" t="str">
         <f t="shared" ref="BT24" si="90">BT$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BU24" s="169"/>
-      <c r="BV24" s="170" t="str">
+      <c r="BU24" s="159"/>
+      <c r="BV24" s="160" t="str">
         <f t="shared" ref="BV24" si="91">BV$8</f>
         <v>C/B</v>
       </c>
-      <c r="BW24" s="171"/>
+      <c r="BW24" s="161"/>
       <c r="BX24" s="66" t="str">
         <f t="shared" ref="BX24:BY24" si="92">BX$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BY24" s="168" t="str">
+      <c r="BY24" s="158" t="str">
         <f t="shared" si="92"/>
         <v>Pur</v>
       </c>
-      <c r="BZ24" s="169"/>
-      <c r="CA24" s="170" t="str">
+      <c r="BZ24" s="159"/>
+      <c r="CA24" s="160" t="str">
         <f t="shared" ref="CA24" si="93">CA$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CB24" s="169"/>
-      <c r="CC24" s="170" t="str">
+      <c r="CB24" s="159"/>
+      <c r="CC24" s="160" t="str">
         <f t="shared" ref="CC24" si="94">CC$8</f>
         <v>C/B</v>
       </c>
-      <c r="CD24" s="171"/>
+      <c r="CD24" s="161"/>
       <c r="CE24" s="66" t="str">
         <f t="shared" ref="CE24:CF24" si="95">CE$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="CF24" s="168" t="str">
+      <c r="CF24" s="158" t="str">
         <f t="shared" si="95"/>
         <v>Pur</v>
       </c>
-      <c r="CG24" s="169"/>
-      <c r="CH24" s="170" t="str">
+      <c r="CG24" s="159"/>
+      <c r="CH24" s="160" t="str">
         <f t="shared" ref="CH24" si="96">CH$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CI24" s="169"/>
-      <c r="CJ24" s="170" t="str">
+      <c r="CI24" s="159"/>
+      <c r="CJ24" s="160" t="str">
         <f t="shared" ref="CJ24" si="97">CJ$8</f>
         <v>C/B</v>
       </c>
-      <c r="CK24" s="171"/>
+      <c r="CK24" s="161"/>
       <c r="CL24" s="66" t="str">
         <f t="shared" ref="CL24:CM24" si="98">CL$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="CM24" s="168" t="str">
+      <c r="CM24" s="158" t="str">
         <f t="shared" si="98"/>
         <v>Pur</v>
       </c>
-      <c r="CN24" s="169"/>
-      <c r="CO24" s="170" t="str">
+      <c r="CN24" s="159"/>
+      <c r="CO24" s="160" t="str">
         <f t="shared" ref="CO24" si="99">CO$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CP24" s="169"/>
-      <c r="CQ24" s="170" t="str">
+      <c r="CP24" s="159"/>
+      <c r="CQ24" s="160" t="str">
         <f t="shared" ref="CQ24" si="100">CQ$8</f>
         <v>C/B</v>
       </c>
-      <c r="CR24" s="171"/>
+      <c r="CR24" s="161"/>
       <c r="CS24" s="66" t="str">
         <f t="shared" ref="CS24" si="101">CS$8</f>
         <v>Inv Days</v>
       </c>
     </row>
-    <row r="25" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
-      <c r="C25" s="174"/>
-      <c r="D25" s="183"/>
-      <c r="E25" s="178"/>
+    <row r="25" spans="1:111" x14ac:dyDescent="0.2">
+      <c r="C25" s="171"/>
+      <c r="D25" s="173"/>
+      <c r="E25" s="168"/>
       <c r="F25" s="39" t="str">
         <f>F9</f>
         <v>Fct</v>
@@ -6641,7 +6641,7 @@
         <v>T/F</v>
       </c>
     </row>
-    <row r="26" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A26" s="68"/>
       <c r="B26" s="68"/>
       <c r="C26" s="93" t="s">
@@ -6964,7 +6964,7 @@
       <c r="DF26" s="69"/>
       <c r="DG26" s="69"/>
     </row>
-    <row r="27" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A27" s="68"/>
       <c r="B27" s="68"/>
       <c r="C27" s="93" t="s">
@@ -7287,7 +7287,7 @@
       <c r="DF27" s="69"/>
       <c r="DG27" s="69"/>
     </row>
-    <row r="28" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A28" s="68"/>
       <c r="B28" s="68"/>
       <c r="C28" s="93" t="s">
@@ -7610,7 +7610,7 @@
       <c r="DF28" s="69"/>
       <c r="DG28" s="69"/>
     </row>
-    <row r="29" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A29" s="68"/>
       <c r="B29" s="68"/>
       <c r="C29" s="93" t="s">
@@ -7933,7 +7933,7 @@
       <c r="DF29" s="69"/>
       <c r="DG29" s="69"/>
     </row>
-    <row r="30" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A30" s="68"/>
       <c r="B30" s="68"/>
       <c r="C30" s="93" t="s">
@@ -8256,7 +8256,7 @@
       <c r="DF30" s="69"/>
       <c r="DG30" s="69"/>
     </row>
-    <row r="31" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A31" s="68"/>
       <c r="B31" s="68"/>
       <c r="C31" s="93" t="s">
@@ -8580,7 +8580,7 @@
       <c r="DF31" s="69"/>
       <c r="DG31" s="69"/>
     </row>
-    <row r="32" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A32" s="68"/>
       <c r="B32" s="68"/>
       <c r="C32" s="93" t="s">
@@ -8904,7 +8904,7 @@
       <c r="DF32" s="69"/>
       <c r="DG32" s="69"/>
     </row>
-    <row r="33" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A33" s="68"/>
       <c r="B33" s="68"/>
       <c r="C33" s="90" t="s">
@@ -9254,7 +9254,7 @@
       <c r="DF33" s="69"/>
       <c r="DG33" s="69"/>
     </row>
-    <row r="34" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A34" s="68"/>
       <c r="B34" s="68"/>
       <c r="C34" s="89" t="s">
@@ -9420,7 +9420,7 @@
       <c r="DF34" s="69"/>
       <c r="DG34" s="69"/>
     </row>
-    <row r="35" spans="1:111" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:111" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="69"/>
       <c r="B35" s="68"/>
       <c r="C35" s="91" t="s">
@@ -9797,7 +9797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:111" s="97" customFormat="1" ht="16" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:111" s="97" customFormat="1" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="C36" s="98"/>
       <c r="D36" s="46"/>
       <c r="E36" s="46"/>
@@ -9999,7 +9999,7 @@
       </c>
       <c r="CS36" s="71"/>
     </row>
-    <row r="37" spans="1:111" s="129" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:111" s="129" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C37" s="130"/>
       <c r="D37" s="131"/>
       <c r="E37" s="131"/>
@@ -10144,7 +10144,7 @@
       <c r="CR37" s="131"/>
       <c r="CS37" s="131"/>
     </row>
-    <row r="38" spans="1:111" s="129" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:111" s="129" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C38" s="130"/>
       <c r="D38" s="131"/>
       <c r="E38" s="131"/>
@@ -10230,7 +10230,7 @@
       <c r="CK38" s="131"/>
       <c r="CL38" s="131"/>
     </row>
-    <row r="39" spans="1:111" ht="18.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:111" ht="18.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C39" s="88"/>
       <c r="H39" s="54"/>
       <c r="I39" s="54"/>
@@ -10312,409 +10312,409 @@
       </c>
       <c r="CL39" s="54"/>
     </row>
-    <row r="40" spans="1:111" ht="16" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="C40" s="172" t="s">
+    <row r="40" spans="1:111" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="C40" s="169" t="s">
         <v>36</v>
       </c>
-      <c r="D40" s="175" t="s">
+      <c r="D40" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="E40" s="176"/>
+      <c r="E40" s="166"/>
       <c r="F40" s="1"/>
-      <c r="G40" s="165">
+      <c r="G40" s="162">
         <f>G$7</f>
         <v>45748</v>
       </c>
-      <c r="H40" s="166"/>
-      <c r="I40" s="166"/>
-      <c r="J40" s="166"/>
-      <c r="K40" s="166"/>
-      <c r="L40" s="166"/>
-      <c r="M40" s="167"/>
-      <c r="N40" s="165">
+      <c r="H40" s="163"/>
+      <c r="I40" s="163"/>
+      <c r="J40" s="163"/>
+      <c r="K40" s="163"/>
+      <c r="L40" s="163"/>
+      <c r="M40" s="164"/>
+      <c r="N40" s="162">
         <f>N$7</f>
         <v>45778</v>
       </c>
-      <c r="O40" s="166"/>
-      <c r="P40" s="166"/>
-      <c r="Q40" s="166"/>
-      <c r="R40" s="166"/>
-      <c r="S40" s="166"/>
-      <c r="T40" s="166"/>
-      <c r="U40" s="165">
+      <c r="O40" s="163"/>
+      <c r="P40" s="163"/>
+      <c r="Q40" s="163"/>
+      <c r="R40" s="163"/>
+      <c r="S40" s="163"/>
+      <c r="T40" s="163"/>
+      <c r="U40" s="162">
         <f>U$7</f>
         <v>45809</v>
       </c>
-      <c r="V40" s="166"/>
-      <c r="W40" s="166"/>
-      <c r="X40" s="166"/>
-      <c r="Y40" s="166"/>
-      <c r="Z40" s="166"/>
-      <c r="AA40" s="167"/>
-      <c r="AB40" s="165">
+      <c r="V40" s="163"/>
+      <c r="W40" s="163"/>
+      <c r="X40" s="163"/>
+      <c r="Y40" s="163"/>
+      <c r="Z40" s="163"/>
+      <c r="AA40" s="164"/>
+      <c r="AB40" s="162">
         <f>AB$7</f>
         <v>45839</v>
       </c>
-      <c r="AC40" s="166"/>
-      <c r="AD40" s="166"/>
-      <c r="AE40" s="166"/>
-      <c r="AF40" s="166"/>
-      <c r="AG40" s="166"/>
-      <c r="AH40" s="167"/>
-      <c r="AI40" s="165">
+      <c r="AC40" s="163"/>
+      <c r="AD40" s="163"/>
+      <c r="AE40" s="163"/>
+      <c r="AF40" s="163"/>
+      <c r="AG40" s="163"/>
+      <c r="AH40" s="164"/>
+      <c r="AI40" s="162">
         <f>AI$7</f>
         <v>45870</v>
       </c>
-      <c r="AJ40" s="166"/>
-      <c r="AK40" s="166"/>
-      <c r="AL40" s="166"/>
-      <c r="AM40" s="166"/>
-      <c r="AN40" s="166"/>
-      <c r="AO40" s="167"/>
-      <c r="AP40" s="165">
+      <c r="AJ40" s="163"/>
+      <c r="AK40" s="163"/>
+      <c r="AL40" s="163"/>
+      <c r="AM40" s="163"/>
+      <c r="AN40" s="163"/>
+      <c r="AO40" s="164"/>
+      <c r="AP40" s="162">
         <f>AP$7</f>
         <v>45901</v>
       </c>
-      <c r="AQ40" s="166"/>
-      <c r="AR40" s="166"/>
-      <c r="AS40" s="166"/>
-      <c r="AT40" s="166"/>
-      <c r="AU40" s="166"/>
-      <c r="AV40" s="167"/>
-      <c r="AW40" s="165">
+      <c r="AQ40" s="163"/>
+      <c r="AR40" s="163"/>
+      <c r="AS40" s="163"/>
+      <c r="AT40" s="163"/>
+      <c r="AU40" s="163"/>
+      <c r="AV40" s="164"/>
+      <c r="AW40" s="162">
         <f>AW$7</f>
         <v>45931</v>
       </c>
-      <c r="AX40" s="166"/>
-      <c r="AY40" s="166"/>
-      <c r="AZ40" s="166"/>
-      <c r="BA40" s="166"/>
-      <c r="BB40" s="166"/>
-      <c r="BC40" s="167"/>
-      <c r="BD40" s="165">
+      <c r="AX40" s="163"/>
+      <c r="AY40" s="163"/>
+      <c r="AZ40" s="163"/>
+      <c r="BA40" s="163"/>
+      <c r="BB40" s="163"/>
+      <c r="BC40" s="164"/>
+      <c r="BD40" s="162">
         <f>BD$7</f>
         <v>45962</v>
       </c>
-      <c r="BE40" s="166"/>
-      <c r="BF40" s="166"/>
-      <c r="BG40" s="166"/>
-      <c r="BH40" s="166"/>
-      <c r="BI40" s="166"/>
-      <c r="BJ40" s="167"/>
-      <c r="BK40" s="165">
+      <c r="BE40" s="163"/>
+      <c r="BF40" s="163"/>
+      <c r="BG40" s="163"/>
+      <c r="BH40" s="163"/>
+      <c r="BI40" s="163"/>
+      <c r="BJ40" s="164"/>
+      <c r="BK40" s="162">
         <f>BK$7</f>
         <v>45992</v>
       </c>
-      <c r="BL40" s="166"/>
-      <c r="BM40" s="166"/>
-      <c r="BN40" s="166"/>
-      <c r="BO40" s="166"/>
-      <c r="BP40" s="166"/>
-      <c r="BQ40" s="167"/>
-      <c r="BR40" s="165">
+      <c r="BL40" s="163"/>
+      <c r="BM40" s="163"/>
+      <c r="BN40" s="163"/>
+      <c r="BO40" s="163"/>
+      <c r="BP40" s="163"/>
+      <c r="BQ40" s="164"/>
+      <c r="BR40" s="162">
         <f>BR$7</f>
         <v>46023</v>
       </c>
-      <c r="BS40" s="166"/>
-      <c r="BT40" s="166"/>
-      <c r="BU40" s="166"/>
-      <c r="BV40" s="166"/>
-      <c r="BW40" s="166"/>
-      <c r="BX40" s="167"/>
-      <c r="BY40" s="165">
+      <c r="BS40" s="163"/>
+      <c r="BT40" s="163"/>
+      <c r="BU40" s="163"/>
+      <c r="BV40" s="163"/>
+      <c r="BW40" s="163"/>
+      <c r="BX40" s="164"/>
+      <c r="BY40" s="162">
         <f>BY$7</f>
         <v>46054</v>
       </c>
-      <c r="BZ40" s="166"/>
-      <c r="CA40" s="166"/>
-      <c r="CB40" s="166"/>
-      <c r="CC40" s="166"/>
-      <c r="CD40" s="166"/>
-      <c r="CE40" s="167"/>
-      <c r="CF40" s="165">
+      <c r="BZ40" s="163"/>
+      <c r="CA40" s="163"/>
+      <c r="CB40" s="163"/>
+      <c r="CC40" s="163"/>
+      <c r="CD40" s="163"/>
+      <c r="CE40" s="164"/>
+      <c r="CF40" s="162">
         <f>CF$7</f>
         <v>46082</v>
       </c>
-      <c r="CG40" s="166"/>
-      <c r="CH40" s="166"/>
-      <c r="CI40" s="166"/>
-      <c r="CJ40" s="166"/>
-      <c r="CK40" s="166"/>
-      <c r="CL40" s="167"/>
-      <c r="CM40" s="165" t="str">
+      <c r="CG40" s="163"/>
+      <c r="CH40" s="163"/>
+      <c r="CI40" s="163"/>
+      <c r="CJ40" s="163"/>
+      <c r="CK40" s="163"/>
+      <c r="CL40" s="164"/>
+      <c r="CM40" s="162" t="str">
         <f>CM$7</f>
         <v>FY26 1H</v>
       </c>
-      <c r="CN40" s="166"/>
-      <c r="CO40" s="166"/>
-      <c r="CP40" s="166"/>
-      <c r="CQ40" s="166"/>
-      <c r="CR40" s="166"/>
-      <c r="CS40" s="167"/>
+      <c r="CN40" s="163"/>
+      <c r="CO40" s="163"/>
+      <c r="CP40" s="163"/>
+      <c r="CQ40" s="163"/>
+      <c r="CR40" s="163"/>
+      <c r="CS40" s="164"/>
     </row>
-    <row r="41" spans="1:111" ht="14.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C41" s="173"/>
-      <c r="D41" s="182" t="s">
+    <row r="41" spans="1:111" ht="14.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C41" s="170"/>
+      <c r="D41" s="172" t="s">
         <v>4</v>
       </c>
-      <c r="E41" s="177" t="s">
+      <c r="E41" s="167" t="s">
         <v>5</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G41" s="168" t="str">
+      <c r="G41" s="158" t="str">
         <f>G$8</f>
         <v>Pur</v>
       </c>
-      <c r="H41" s="169"/>
-      <c r="I41" s="170" t="str">
+      <c r="H41" s="159"/>
+      <c r="I41" s="160" t="str">
         <f>I$8</f>
         <v>Consumption</v>
       </c>
-      <c r="J41" s="169"/>
-      <c r="K41" s="170" t="str">
+      <c r="J41" s="159"/>
+      <c r="K41" s="160" t="str">
         <f>K$8</f>
         <v>C/B</v>
       </c>
-      <c r="L41" s="171"/>
+      <c r="L41" s="161"/>
       <c r="M41" s="66" t="str">
         <f>M$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="N41" s="168" t="str">
+      <c r="N41" s="158" t="str">
         <f>N$8</f>
         <v>Pur</v>
       </c>
-      <c r="O41" s="169"/>
-      <c r="P41" s="170" t="str">
+      <c r="O41" s="159"/>
+      <c r="P41" s="160" t="str">
         <f>P$8</f>
         <v>Consumption</v>
       </c>
-      <c r="Q41" s="169"/>
-      <c r="R41" s="170" t="str">
+      <c r="Q41" s="159"/>
+      <c r="R41" s="160" t="str">
         <f>R$8</f>
         <v>C/B</v>
       </c>
-      <c r="S41" s="171"/>
+      <c r="S41" s="161"/>
       <c r="T41" s="66" t="str">
         <f t="shared" ref="T41" si="170">T$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="U41" s="168" t="str">
+      <c r="U41" s="158" t="str">
         <f t="shared" ref="U41" si="171">U$8</f>
         <v>Pur</v>
       </c>
-      <c r="V41" s="169"/>
-      <c r="W41" s="170" t="str">
+      <c r="V41" s="159"/>
+      <c r="W41" s="160" t="str">
         <f t="shared" ref="W41" si="172">W$8</f>
         <v>Consumption</v>
       </c>
-      <c r="X41" s="169"/>
-      <c r="Y41" s="170" t="str">
+      <c r="X41" s="159"/>
+      <c r="Y41" s="160" t="str">
         <f t="shared" ref="Y41" si="173">Y$8</f>
         <v>C/B</v>
       </c>
-      <c r="Z41" s="171"/>
+      <c r="Z41" s="161"/>
       <c r="AA41" s="66" t="str">
         <f t="shared" ref="AA41:AB41" si="174">AA$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AB41" s="168" t="str">
+      <c r="AB41" s="158" t="str">
         <f t="shared" si="174"/>
         <v>Pur</v>
       </c>
-      <c r="AC41" s="169"/>
-      <c r="AD41" s="170" t="str">
+      <c r="AC41" s="159"/>
+      <c r="AD41" s="160" t="str">
         <f t="shared" ref="AD41" si="175">AD$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AE41" s="169"/>
-      <c r="AF41" s="170" t="str">
+      <c r="AE41" s="159"/>
+      <c r="AF41" s="160" t="str">
         <f t="shared" ref="AF41" si="176">AF$8</f>
         <v>C/B</v>
       </c>
-      <c r="AG41" s="171"/>
+      <c r="AG41" s="161"/>
       <c r="AH41" s="66" t="str">
         <f t="shared" ref="AH41:AI41" si="177">AH$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AI41" s="168" t="str">
+      <c r="AI41" s="158" t="str">
         <f t="shared" si="177"/>
         <v>Pur</v>
       </c>
-      <c r="AJ41" s="169"/>
-      <c r="AK41" s="170" t="str">
+      <c r="AJ41" s="159"/>
+      <c r="AK41" s="160" t="str">
         <f t="shared" ref="AK41" si="178">AK$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AL41" s="169"/>
-      <c r="AM41" s="170" t="str">
+      <c r="AL41" s="159"/>
+      <c r="AM41" s="160" t="str">
         <f t="shared" ref="AM41" si="179">AM$8</f>
         <v>C/B</v>
       </c>
-      <c r="AN41" s="169"/>
+      <c r="AN41" s="159"/>
       <c r="AO41" s="83" t="str">
         <f t="shared" ref="AO41:AP41" si="180">AO$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AP41" s="168" t="str">
+      <c r="AP41" s="158" t="str">
         <f t="shared" si="180"/>
         <v>Pur</v>
       </c>
-      <c r="AQ41" s="169"/>
-      <c r="AR41" s="170" t="str">
+      <c r="AQ41" s="159"/>
+      <c r="AR41" s="160" t="str">
         <f t="shared" ref="AR41" si="181">AR$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AS41" s="169"/>
-      <c r="AT41" s="170" t="str">
+      <c r="AS41" s="159"/>
+      <c r="AT41" s="160" t="str">
         <f t="shared" ref="AT41" si="182">AT$8</f>
         <v>C/B</v>
       </c>
-      <c r="AU41" s="169"/>
+      <c r="AU41" s="159"/>
       <c r="AV41" s="66" t="str">
         <f t="shared" ref="AV41:AW41" si="183">AV$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AW41" s="168" t="str">
+      <c r="AW41" s="158" t="str">
         <f t="shared" si="183"/>
         <v>Pur</v>
       </c>
-      <c r="AX41" s="169"/>
-      <c r="AY41" s="170" t="str">
+      <c r="AX41" s="159"/>
+      <c r="AY41" s="160" t="str">
         <f t="shared" ref="AY41" si="184">AY$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AZ41" s="169"/>
-      <c r="BA41" s="170" t="str">
+      <c r="AZ41" s="159"/>
+      <c r="BA41" s="160" t="str">
         <f t="shared" ref="BA41" si="185">BA$8</f>
         <v>C/B</v>
       </c>
-      <c r="BB41" s="169"/>
+      <c r="BB41" s="159"/>
       <c r="BC41" s="66" t="str">
         <f t="shared" ref="BC41:BD41" si="186">BC$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BD41" s="168" t="str">
+      <c r="BD41" s="158" t="str">
         <f t="shared" si="186"/>
         <v>Pur</v>
       </c>
-      <c r="BE41" s="169"/>
-      <c r="BF41" s="170" t="str">
+      <c r="BE41" s="159"/>
+      <c r="BF41" s="160" t="str">
         <f t="shared" ref="BF41" si="187">BF$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BG41" s="169"/>
-      <c r="BH41" s="170" t="str">
+      <c r="BG41" s="159"/>
+      <c r="BH41" s="160" t="str">
         <f t="shared" ref="BH41" si="188">BH$8</f>
         <v>C/B</v>
       </c>
-      <c r="BI41" s="169"/>
+      <c r="BI41" s="159"/>
       <c r="BJ41" s="66" t="str">
         <f t="shared" ref="BJ41:BK41" si="189">BJ$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BK41" s="168" t="str">
+      <c r="BK41" s="158" t="str">
         <f t="shared" si="189"/>
         <v>Pur</v>
       </c>
-      <c r="BL41" s="169"/>
-      <c r="BM41" s="170" t="str">
+      <c r="BL41" s="159"/>
+      <c r="BM41" s="160" t="str">
         <f t="shared" ref="BM41" si="190">BM$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BN41" s="169"/>
-      <c r="BO41" s="170" t="str">
+      <c r="BN41" s="159"/>
+      <c r="BO41" s="160" t="str">
         <f t="shared" ref="BO41" si="191">BO$8</f>
         <v>C/B</v>
       </c>
-      <c r="BP41" s="169"/>
+      <c r="BP41" s="159"/>
       <c r="BQ41" s="66" t="str">
         <f t="shared" ref="BQ41:BR41" si="192">BQ$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BR41" s="168" t="str">
+      <c r="BR41" s="158" t="str">
         <f t="shared" si="192"/>
         <v>Pur</v>
       </c>
-      <c r="BS41" s="169"/>
-      <c r="BT41" s="170" t="str">
+      <c r="BS41" s="159"/>
+      <c r="BT41" s="160" t="str">
         <f t="shared" ref="BT41" si="193">BT$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BU41" s="169"/>
-      <c r="BV41" s="170" t="str">
+      <c r="BU41" s="159"/>
+      <c r="BV41" s="160" t="str">
         <f t="shared" ref="BV41" si="194">BV$8</f>
         <v>C/B</v>
       </c>
-      <c r="BW41" s="169"/>
+      <c r="BW41" s="159"/>
       <c r="BX41" s="66" t="str">
         <f t="shared" ref="BX41:BY41" si="195">BX$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BY41" s="168" t="str">
+      <c r="BY41" s="158" t="str">
         <f t="shared" si="195"/>
         <v>Pur</v>
       </c>
-      <c r="BZ41" s="169"/>
-      <c r="CA41" s="170" t="str">
+      <c r="BZ41" s="159"/>
+      <c r="CA41" s="160" t="str">
         <f t="shared" ref="CA41" si="196">CA$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CB41" s="169"/>
-      <c r="CC41" s="170" t="str">
+      <c r="CB41" s="159"/>
+      <c r="CC41" s="160" t="str">
         <f t="shared" ref="CC41" si="197">CC$8</f>
         <v>C/B</v>
       </c>
-      <c r="CD41" s="169"/>
+      <c r="CD41" s="159"/>
       <c r="CE41" s="66" t="str">
         <f t="shared" ref="CE41:CF41" si="198">CE$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="CF41" s="168" t="str">
+      <c r="CF41" s="158" t="str">
         <f t="shared" si="198"/>
         <v>Pur</v>
       </c>
-      <c r="CG41" s="169"/>
-      <c r="CH41" s="170" t="str">
+      <c r="CG41" s="159"/>
+      <c r="CH41" s="160" t="str">
         <f t="shared" ref="CH41" si="199">CH$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CI41" s="169"/>
-      <c r="CJ41" s="170" t="str">
+      <c r="CI41" s="159"/>
+      <c r="CJ41" s="160" t="str">
         <f t="shared" ref="CJ41" si="200">CJ$8</f>
         <v>C/B</v>
       </c>
-      <c r="CK41" s="169"/>
+      <c r="CK41" s="159"/>
       <c r="CL41" s="66" t="str">
         <f t="shared" ref="CL41:CM41" si="201">CL$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="CM41" s="168" t="str">
+      <c r="CM41" s="158" t="str">
         <f t="shared" si="201"/>
         <v>Pur</v>
       </c>
-      <c r="CN41" s="169"/>
-      <c r="CO41" s="170" t="str">
+      <c r="CN41" s="159"/>
+      <c r="CO41" s="160" t="str">
         <f t="shared" ref="CO41" si="202">CO$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CP41" s="169"/>
-      <c r="CQ41" s="170" t="str">
+      <c r="CP41" s="159"/>
+      <c r="CQ41" s="160" t="str">
         <f t="shared" ref="CQ41" si="203">CQ$8</f>
         <v>C/B</v>
       </c>
-      <c r="CR41" s="169"/>
+      <c r="CR41" s="159"/>
       <c r="CS41" s="66" t="str">
         <f t="shared" ref="CS41" si="204">CS$8</f>
         <v>Inv Days</v>
       </c>
     </row>
-    <row r="42" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
-      <c r="C42" s="174"/>
-      <c r="D42" s="183"/>
-      <c r="E42" s="178"/>
+    <row r="42" spans="1:111" x14ac:dyDescent="0.2">
+      <c r="C42" s="171"/>
+      <c r="D42" s="173"/>
+      <c r="E42" s="168"/>
       <c r="F42" s="2" t="str">
         <f>F9</f>
         <v>Fct</v>
@@ -11084,7 +11084,7 @@
         <v>T/F</v>
       </c>
     </row>
-    <row r="43" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A43" s="68"/>
       <c r="B43" s="68"/>
       <c r="C43" s="93" t="s">
@@ -11397,7 +11397,7 @@
         <v>98.928215486693972</v>
       </c>
     </row>
-    <row r="44" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A44" s="68"/>
       <c r="B44" s="68"/>
       <c r="C44" s="93" t="s">
@@ -11710,7 +11710,7 @@
         <v>141.33432467650735</v>
       </c>
     </row>
-    <row r="45" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A45" s="68"/>
       <c r="B45" s="68"/>
       <c r="C45" s="93" t="s">
@@ -12023,7 +12023,7 @@
         <v>12.434154789498088</v>
       </c>
     </row>
-    <row r="46" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A46" s="68"/>
       <c r="B46" s="68"/>
       <c r="C46" s="93" t="s">
@@ -12331,7 +12331,7 @@
         <v>-8.3585910743191132</v>
       </c>
     </row>
-    <row r="47" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A47" s="68"/>
       <c r="B47" s="68"/>
       <c r="C47" s="93" t="s">
@@ -12644,7 +12644,7 @@
         <v>101.31338455310407</v>
       </c>
     </row>
-    <row r="48" spans="1:111" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:111" x14ac:dyDescent="0.2">
       <c r="A48" s="68"/>
       <c r="B48" s="68"/>
       <c r="C48" s="93" t="s">
@@ -12957,7 +12957,7 @@
         <v>182.69611863312124</v>
       </c>
     </row>
-    <row r="49" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A49" s="68"/>
       <c r="B49" s="68"/>
       <c r="C49" s="93" t="s">
@@ -13270,7 +13270,7 @@
         <v>44.336478079586122</v>
       </c>
     </row>
-    <row r="50" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A50" s="68"/>
       <c r="B50" s="68"/>
       <c r="C50" s="93" t="s">
@@ -13511,7 +13511,7 @@
         <v>-3201.4510268140962</v>
       </c>
     </row>
-    <row r="51" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A51" s="68"/>
       <c r="B51" s="68"/>
       <c r="C51" s="93" t="s">
@@ -13781,7 +13781,7 @@
       </c>
       <c r="CS51" s="15"/>
     </row>
-    <row r="52" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A52" s="68"/>
       <c r="B52" s="68"/>
       <c r="C52" s="90" t="s">
@@ -14119,7 +14119,7 @@
       </c>
       <c r="CS52" s="82"/>
     </row>
-    <row r="53" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A53" s="68"/>
       <c r="B53" s="68"/>
       <c r="C53" s="89" t="s">
@@ -14272,7 +14272,7 @@
       <c r="CR53" s="51"/>
       <c r="CS53" s="18"/>
     </row>
-    <row r="54" spans="1:97" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:97" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="69"/>
       <c r="B54" s="68"/>
       <c r="C54" s="91" t="s">
@@ -14649,7 +14649,7 @@
         <v>50.936902266775576</v>
       </c>
     </row>
-    <row r="55" spans="1:97" s="97" customFormat="1" ht="16" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:97" s="97" customFormat="1" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="C55" s="98"/>
       <c r="D55" s="46"/>
       <c r="E55" s="46"/>
@@ -14785,7 +14785,7 @@
       </c>
       <c r="CS55" s="101"/>
     </row>
-    <row r="56" spans="1:97" s="97" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:97" s="97" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C56" s="98"/>
       <c r="D56" s="46"/>
       <c r="E56" s="46"/>
@@ -14874,7 +14874,7 @@
       <c r="CK56" s="46"/>
       <c r="CL56" s="46"/>
     </row>
-    <row r="57" spans="1:97" s="84" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:97" s="84" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B57" s="97"/>
       <c r="C57" s="94"/>
       <c r="D57" s="85"/>
@@ -14965,7 +14965,7 @@
       <c r="CK57" s="121"/>
       <c r="CL57" s="120"/>
     </row>
-    <row r="58" spans="1:97" ht="18.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:97" ht="18.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C58" s="88"/>
       <c r="H58" s="54"/>
       <c r="I58" s="54"/>
@@ -15047,409 +15047,409 @@
       </c>
       <c r="CL58" s="54"/>
     </row>
-    <row r="59" spans="1:97" ht="15" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="C59" s="172" t="s">
+    <row r="59" spans="1:97" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="C59" s="169" t="s">
         <v>46</v>
       </c>
-      <c r="D59" s="175" t="s">
+      <c r="D59" s="165" t="s">
         <v>2</v>
       </c>
-      <c r="E59" s="176"/>
+      <c r="E59" s="166"/>
       <c r="F59" s="1"/>
-      <c r="G59" s="165">
+      <c r="G59" s="162">
         <f>G$7</f>
         <v>45748</v>
       </c>
-      <c r="H59" s="166"/>
-      <c r="I59" s="166"/>
-      <c r="J59" s="166"/>
-      <c r="K59" s="166"/>
-      <c r="L59" s="166"/>
-      <c r="M59" s="167"/>
-      <c r="N59" s="165">
+      <c r="H59" s="163"/>
+      <c r="I59" s="163"/>
+      <c r="J59" s="163"/>
+      <c r="K59" s="163"/>
+      <c r="L59" s="163"/>
+      <c r="M59" s="164"/>
+      <c r="N59" s="162">
         <f>N$7</f>
         <v>45778</v>
       </c>
-      <c r="O59" s="166"/>
-      <c r="P59" s="166"/>
-      <c r="Q59" s="166"/>
-      <c r="R59" s="166"/>
-      <c r="S59" s="166"/>
-      <c r="T59" s="166"/>
-      <c r="U59" s="165">
+      <c r="O59" s="163"/>
+      <c r="P59" s="163"/>
+      <c r="Q59" s="163"/>
+      <c r="R59" s="163"/>
+      <c r="S59" s="163"/>
+      <c r="T59" s="163"/>
+      <c r="U59" s="162">
         <f>U$7</f>
         <v>45809</v>
       </c>
-      <c r="V59" s="166"/>
-      <c r="W59" s="166"/>
-      <c r="X59" s="166"/>
-      <c r="Y59" s="166"/>
-      <c r="Z59" s="166"/>
-      <c r="AA59" s="167"/>
-      <c r="AB59" s="165">
+      <c r="V59" s="163"/>
+      <c r="W59" s="163"/>
+      <c r="X59" s="163"/>
+      <c r="Y59" s="163"/>
+      <c r="Z59" s="163"/>
+      <c r="AA59" s="164"/>
+      <c r="AB59" s="162">
         <f>AB$7</f>
         <v>45839</v>
       </c>
-      <c r="AC59" s="166"/>
-      <c r="AD59" s="166"/>
-      <c r="AE59" s="166"/>
-      <c r="AF59" s="166"/>
-      <c r="AG59" s="166"/>
-      <c r="AH59" s="167"/>
-      <c r="AI59" s="165">
+      <c r="AC59" s="163"/>
+      <c r="AD59" s="163"/>
+      <c r="AE59" s="163"/>
+      <c r="AF59" s="163"/>
+      <c r="AG59" s="163"/>
+      <c r="AH59" s="164"/>
+      <c r="AI59" s="162">
         <f>AI$7</f>
         <v>45870</v>
       </c>
-      <c r="AJ59" s="166"/>
-      <c r="AK59" s="166"/>
-      <c r="AL59" s="166"/>
-      <c r="AM59" s="166"/>
-      <c r="AN59" s="166"/>
-      <c r="AO59" s="167"/>
-      <c r="AP59" s="165">
+      <c r="AJ59" s="163"/>
+      <c r="AK59" s="163"/>
+      <c r="AL59" s="163"/>
+      <c r="AM59" s="163"/>
+      <c r="AN59" s="163"/>
+      <c r="AO59" s="164"/>
+      <c r="AP59" s="162">
         <f>AP$7</f>
         <v>45901</v>
       </c>
-      <c r="AQ59" s="166"/>
-      <c r="AR59" s="166"/>
-      <c r="AS59" s="166"/>
-      <c r="AT59" s="166"/>
-      <c r="AU59" s="166"/>
-      <c r="AV59" s="167"/>
-      <c r="AW59" s="165">
+      <c r="AQ59" s="163"/>
+      <c r="AR59" s="163"/>
+      <c r="AS59" s="163"/>
+      <c r="AT59" s="163"/>
+      <c r="AU59" s="163"/>
+      <c r="AV59" s="164"/>
+      <c r="AW59" s="162">
         <f>AW$7</f>
         <v>45931</v>
       </c>
-      <c r="AX59" s="166"/>
-      <c r="AY59" s="166"/>
-      <c r="AZ59" s="166"/>
-      <c r="BA59" s="166"/>
-      <c r="BB59" s="166"/>
-      <c r="BC59" s="167"/>
-      <c r="BD59" s="165">
+      <c r="AX59" s="163"/>
+      <c r="AY59" s="163"/>
+      <c r="AZ59" s="163"/>
+      <c r="BA59" s="163"/>
+      <c r="BB59" s="163"/>
+      <c r="BC59" s="164"/>
+      <c r="BD59" s="162">
         <f>BD$7</f>
         <v>45962</v>
       </c>
-      <c r="BE59" s="166"/>
-      <c r="BF59" s="166"/>
-      <c r="BG59" s="166"/>
-      <c r="BH59" s="166"/>
-      <c r="BI59" s="166"/>
-      <c r="BJ59" s="167"/>
-      <c r="BK59" s="165">
+      <c r="BE59" s="163"/>
+      <c r="BF59" s="163"/>
+      <c r="BG59" s="163"/>
+      <c r="BH59" s="163"/>
+      <c r="BI59" s="163"/>
+      <c r="BJ59" s="164"/>
+      <c r="BK59" s="162">
         <f>BK$7</f>
         <v>45992</v>
       </c>
-      <c r="BL59" s="166"/>
-      <c r="BM59" s="166"/>
-      <c r="BN59" s="166"/>
-      <c r="BO59" s="166"/>
-      <c r="BP59" s="166"/>
-      <c r="BQ59" s="167"/>
-      <c r="BR59" s="165">
+      <c r="BL59" s="163"/>
+      <c r="BM59" s="163"/>
+      <c r="BN59" s="163"/>
+      <c r="BO59" s="163"/>
+      <c r="BP59" s="163"/>
+      <c r="BQ59" s="164"/>
+      <c r="BR59" s="162">
         <f>BR$7</f>
         <v>46023</v>
       </c>
-      <c r="BS59" s="166"/>
-      <c r="BT59" s="166"/>
-      <c r="BU59" s="166"/>
-      <c r="BV59" s="166"/>
-      <c r="BW59" s="166"/>
-      <c r="BX59" s="167"/>
-      <c r="BY59" s="165">
+      <c r="BS59" s="163"/>
+      <c r="BT59" s="163"/>
+      <c r="BU59" s="163"/>
+      <c r="BV59" s="163"/>
+      <c r="BW59" s="163"/>
+      <c r="BX59" s="164"/>
+      <c r="BY59" s="162">
         <f>BY$7</f>
         <v>46054</v>
       </c>
-      <c r="BZ59" s="166"/>
-      <c r="CA59" s="166"/>
-      <c r="CB59" s="166"/>
-      <c r="CC59" s="166"/>
-      <c r="CD59" s="166"/>
-      <c r="CE59" s="167"/>
-      <c r="CF59" s="165">
+      <c r="BZ59" s="163"/>
+      <c r="CA59" s="163"/>
+      <c r="CB59" s="163"/>
+      <c r="CC59" s="163"/>
+      <c r="CD59" s="163"/>
+      <c r="CE59" s="164"/>
+      <c r="CF59" s="162">
         <f>CF$7</f>
         <v>46082</v>
       </c>
-      <c r="CG59" s="166"/>
-      <c r="CH59" s="166"/>
-      <c r="CI59" s="166"/>
-      <c r="CJ59" s="166"/>
-      <c r="CK59" s="166"/>
-      <c r="CL59" s="167"/>
-      <c r="CM59" s="165" t="str">
+      <c r="CG59" s="163"/>
+      <c r="CH59" s="163"/>
+      <c r="CI59" s="163"/>
+      <c r="CJ59" s="163"/>
+      <c r="CK59" s="163"/>
+      <c r="CL59" s="164"/>
+      <c r="CM59" s="162" t="str">
         <f>CM$7</f>
         <v>FY26 1H</v>
       </c>
-      <c r="CN59" s="166"/>
-      <c r="CO59" s="166"/>
-      <c r="CP59" s="166"/>
-      <c r="CQ59" s="166"/>
-      <c r="CR59" s="166"/>
-      <c r="CS59" s="167"/>
+      <c r="CN59" s="163"/>
+      <c r="CO59" s="163"/>
+      <c r="CP59" s="163"/>
+      <c r="CQ59" s="163"/>
+      <c r="CR59" s="163"/>
+      <c r="CS59" s="164"/>
     </row>
-    <row r="60" spans="1:97" ht="14.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C60" s="173"/>
-      <c r="D60" s="182" t="s">
+    <row r="60" spans="1:97" ht="14.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C60" s="170"/>
+      <c r="D60" s="172" t="s">
         <v>4</v>
       </c>
-      <c r="E60" s="177" t="s">
+      <c r="E60" s="167" t="s">
         <v>47</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G60" s="168" t="str">
+      <c r="G60" s="158" t="str">
         <f>G$8</f>
         <v>Pur</v>
       </c>
-      <c r="H60" s="169"/>
-      <c r="I60" s="170" t="str">
+      <c r="H60" s="159"/>
+      <c r="I60" s="160" t="str">
         <f>I$8</f>
         <v>Consumption</v>
       </c>
-      <c r="J60" s="169"/>
-      <c r="K60" s="170" t="str">
+      <c r="J60" s="159"/>
+      <c r="K60" s="160" t="str">
         <f>K$8</f>
         <v>C/B</v>
       </c>
-      <c r="L60" s="171"/>
+      <c r="L60" s="161"/>
       <c r="M60" s="66" t="str">
         <f>M$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="N60" s="168" t="str">
+      <c r="N60" s="158" t="str">
         <f>N$8</f>
         <v>Pur</v>
       </c>
-      <c r="O60" s="169"/>
-      <c r="P60" s="170" t="str">
+      <c r="O60" s="159"/>
+      <c r="P60" s="160" t="str">
         <f>P$8</f>
         <v>Consumption</v>
       </c>
-      <c r="Q60" s="169"/>
-      <c r="R60" s="170" t="str">
+      <c r="Q60" s="159"/>
+      <c r="R60" s="160" t="str">
         <f>R$8</f>
         <v>C/B</v>
       </c>
-      <c r="S60" s="171"/>
+      <c r="S60" s="161"/>
       <c r="T60" s="66" t="str">
         <f t="shared" ref="T60" si="278">T$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="U60" s="168" t="str">
+      <c r="U60" s="158" t="str">
         <f t="shared" ref="U60" si="279">U$8</f>
         <v>Pur</v>
       </c>
-      <c r="V60" s="169"/>
-      <c r="W60" s="170" t="str">
+      <c r="V60" s="159"/>
+      <c r="W60" s="160" t="str">
         <f t="shared" ref="W60" si="280">W$8</f>
         <v>Consumption</v>
       </c>
-      <c r="X60" s="169"/>
-      <c r="Y60" s="170" t="str">
+      <c r="X60" s="159"/>
+      <c r="Y60" s="160" t="str">
         <f t="shared" ref="Y60" si="281">Y$8</f>
         <v>C/B</v>
       </c>
-      <c r="Z60" s="171"/>
+      <c r="Z60" s="161"/>
       <c r="AA60" s="66" t="str">
         <f t="shared" ref="AA60:AB60" si="282">AA$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AB60" s="168" t="str">
+      <c r="AB60" s="158" t="str">
         <f t="shared" si="282"/>
         <v>Pur</v>
       </c>
-      <c r="AC60" s="169"/>
-      <c r="AD60" s="170" t="str">
+      <c r="AC60" s="159"/>
+      <c r="AD60" s="160" t="str">
         <f t="shared" ref="AD60" si="283">AD$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AE60" s="169"/>
-      <c r="AF60" s="170" t="str">
+      <c r="AE60" s="159"/>
+      <c r="AF60" s="160" t="str">
         <f t="shared" ref="AF60" si="284">AF$8</f>
         <v>C/B</v>
       </c>
-      <c r="AG60" s="171"/>
+      <c r="AG60" s="161"/>
       <c r="AH60" s="66" t="str">
         <f t="shared" ref="AH60:AI60" si="285">AH$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AI60" s="168" t="str">
+      <c r="AI60" s="158" t="str">
         <f t="shared" si="285"/>
         <v>Pur</v>
       </c>
-      <c r="AJ60" s="169"/>
-      <c r="AK60" s="170" t="str">
+      <c r="AJ60" s="159"/>
+      <c r="AK60" s="160" t="str">
         <f t="shared" ref="AK60" si="286">AK$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AL60" s="169"/>
-      <c r="AM60" s="170" t="str">
+      <c r="AL60" s="159"/>
+      <c r="AM60" s="160" t="str">
         <f t="shared" ref="AM60" si="287">AM$8</f>
         <v>C/B</v>
       </c>
-      <c r="AN60" s="171"/>
+      <c r="AN60" s="161"/>
       <c r="AO60" s="66" t="str">
         <f t="shared" ref="AO60:AP60" si="288">AO$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AP60" s="168" t="str">
+      <c r="AP60" s="158" t="str">
         <f t="shared" si="288"/>
         <v>Pur</v>
       </c>
-      <c r="AQ60" s="169"/>
-      <c r="AR60" s="170" t="str">
+      <c r="AQ60" s="159"/>
+      <c r="AR60" s="160" t="str">
         <f t="shared" ref="AR60" si="289">AR$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AS60" s="169"/>
-      <c r="AT60" s="170" t="str">
+      <c r="AS60" s="159"/>
+      <c r="AT60" s="160" t="str">
         <f t="shared" ref="AT60" si="290">AT$8</f>
         <v>C/B</v>
       </c>
-      <c r="AU60" s="171"/>
+      <c r="AU60" s="161"/>
       <c r="AV60" s="66" t="str">
         <f t="shared" ref="AV60:AW60" si="291">AV$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AW60" s="168" t="str">
+      <c r="AW60" s="158" t="str">
         <f t="shared" si="291"/>
         <v>Pur</v>
       </c>
-      <c r="AX60" s="169"/>
-      <c r="AY60" s="170" t="str">
+      <c r="AX60" s="159"/>
+      <c r="AY60" s="160" t="str">
         <f t="shared" ref="AY60" si="292">AY$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AZ60" s="169"/>
-      <c r="BA60" s="170" t="str">
+      <c r="AZ60" s="159"/>
+      <c r="BA60" s="160" t="str">
         <f t="shared" ref="BA60" si="293">BA$8</f>
         <v>C/B</v>
       </c>
-      <c r="BB60" s="171"/>
+      <c r="BB60" s="161"/>
       <c r="BC60" s="66" t="str">
         <f t="shared" ref="BC60:BD60" si="294">BC$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BD60" s="168" t="str">
+      <c r="BD60" s="158" t="str">
         <f t="shared" si="294"/>
         <v>Pur</v>
       </c>
-      <c r="BE60" s="169"/>
-      <c r="BF60" s="170" t="str">
+      <c r="BE60" s="159"/>
+      <c r="BF60" s="160" t="str">
         <f t="shared" ref="BF60" si="295">BF$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BG60" s="169"/>
-      <c r="BH60" s="170" t="str">
+      <c r="BG60" s="159"/>
+      <c r="BH60" s="160" t="str">
         <f t="shared" ref="BH60" si="296">BH$8</f>
         <v>C/B</v>
       </c>
-      <c r="BI60" s="171"/>
+      <c r="BI60" s="161"/>
       <c r="BJ60" s="66" t="str">
         <f t="shared" ref="BJ60:BK60" si="297">BJ$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BK60" s="168" t="str">
+      <c r="BK60" s="158" t="str">
         <f t="shared" si="297"/>
         <v>Pur</v>
       </c>
-      <c r="BL60" s="169"/>
-      <c r="BM60" s="170" t="str">
+      <c r="BL60" s="159"/>
+      <c r="BM60" s="160" t="str">
         <f t="shared" ref="BM60" si="298">BM$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BN60" s="169"/>
-      <c r="BO60" s="170" t="str">
+      <c r="BN60" s="159"/>
+      <c r="BO60" s="160" t="str">
         <f t="shared" ref="BO60" si="299">BO$8</f>
         <v>C/B</v>
       </c>
-      <c r="BP60" s="171"/>
+      <c r="BP60" s="161"/>
       <c r="BQ60" s="66" t="str">
         <f t="shared" ref="BQ60:BR60" si="300">BQ$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BR60" s="168" t="str">
+      <c r="BR60" s="158" t="str">
         <f t="shared" si="300"/>
         <v>Pur</v>
       </c>
-      <c r="BS60" s="169"/>
-      <c r="BT60" s="170" t="str">
+      <c r="BS60" s="159"/>
+      <c r="BT60" s="160" t="str">
         <f t="shared" ref="BT60" si="301">BT$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BU60" s="169"/>
-      <c r="BV60" s="170" t="str">
+      <c r="BU60" s="159"/>
+      <c r="BV60" s="160" t="str">
         <f t="shared" ref="BV60" si="302">BV$8</f>
         <v>C/B</v>
       </c>
-      <c r="BW60" s="171"/>
+      <c r="BW60" s="161"/>
       <c r="BX60" s="66" t="str">
         <f t="shared" ref="BX60:BY60" si="303">BX$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BY60" s="168" t="str">
+      <c r="BY60" s="158" t="str">
         <f t="shared" si="303"/>
         <v>Pur</v>
       </c>
-      <c r="BZ60" s="169"/>
-      <c r="CA60" s="170" t="str">
+      <c r="BZ60" s="159"/>
+      <c r="CA60" s="160" t="str">
         <f t="shared" ref="CA60" si="304">CA$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CB60" s="169"/>
-      <c r="CC60" s="170" t="str">
+      <c r="CB60" s="159"/>
+      <c r="CC60" s="160" t="str">
         <f t="shared" ref="CC60" si="305">CC$8</f>
         <v>C/B</v>
       </c>
-      <c r="CD60" s="171"/>
+      <c r="CD60" s="161"/>
       <c r="CE60" s="66" t="str">
         <f t="shared" ref="CE60:CF60" si="306">CE$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="CF60" s="168" t="str">
+      <c r="CF60" s="158" t="str">
         <f t="shared" si="306"/>
         <v>Pur</v>
       </c>
-      <c r="CG60" s="169"/>
-      <c r="CH60" s="170" t="str">
+      <c r="CG60" s="159"/>
+      <c r="CH60" s="160" t="str">
         <f t="shared" ref="CH60" si="307">CH$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CI60" s="169"/>
-      <c r="CJ60" s="170" t="str">
+      <c r="CI60" s="159"/>
+      <c r="CJ60" s="160" t="str">
         <f t="shared" ref="CJ60" si="308">CJ$8</f>
         <v>C/B</v>
       </c>
-      <c r="CK60" s="171"/>
+      <c r="CK60" s="161"/>
       <c r="CL60" s="66" t="str">
         <f t="shared" ref="CL60:CM60" si="309">CL$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="CM60" s="168" t="str">
+      <c r="CM60" s="158" t="str">
         <f t="shared" si="309"/>
         <v>Pur</v>
       </c>
-      <c r="CN60" s="169"/>
-      <c r="CO60" s="170" t="str">
+      <c r="CN60" s="159"/>
+      <c r="CO60" s="160" t="str">
         <f t="shared" ref="CO60" si="310">CO$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CP60" s="169"/>
-      <c r="CQ60" s="170" t="str">
+      <c r="CP60" s="159"/>
+      <c r="CQ60" s="160" t="str">
         <f t="shared" ref="CQ60" si="311">CQ$8</f>
         <v>C/B</v>
       </c>
-      <c r="CR60" s="171"/>
+      <c r="CR60" s="161"/>
       <c r="CS60" s="66" t="str">
         <f t="shared" ref="CS60" si="312">CS$8</f>
         <v>Inv Days</v>
       </c>
     </row>
-    <row r="61" spans="1:97" ht="20.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C61" s="174"/>
-      <c r="D61" s="183"/>
-      <c r="E61" s="178"/>
+    <row r="61" spans="1:97" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C61" s="171"/>
+      <c r="D61" s="173"/>
+      <c r="E61" s="168"/>
       <c r="F61" s="2" t="str">
         <f>F42</f>
         <v>Fct</v>
@@ -15819,7 +15819,7 @@
         <v>T/F</v>
       </c>
     </row>
-    <row r="62" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A62" s="68"/>
       <c r="B62" s="68"/>
       <c r="C62" s="93" t="s">
@@ -16130,7 +16130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A63" s="68"/>
       <c r="B63" s="68"/>
       <c r="C63" s="93" t="s">
@@ -16441,7 +16441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A64" s="68"/>
       <c r="B64" s="68"/>
       <c r="C64" s="93" t="s">
@@ -16752,7 +16752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A65" s="68"/>
       <c r="B65" s="68"/>
       <c r="C65" s="93" t="s">
@@ -17063,7 +17063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A66" s="68"/>
       <c r="B66" s="68"/>
       <c r="C66" s="93" t="s">
@@ -17374,7 +17374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A67" s="68"/>
       <c r="B67" s="68"/>
       <c r="C67" s="93" t="s">
@@ -17685,7 +17685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A68" s="68"/>
       <c r="B68" s="68"/>
       <c r="C68" s="93" t="s">
@@ -17948,7 +17948,7 @@
       <c r="CR68" s="13"/>
       <c r="CS68" s="15"/>
     </row>
-    <row r="69" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A69" s="68"/>
       <c r="B69" s="68"/>
       <c r="C69" s="93" t="s">
@@ -18166,7 +18166,7 @@
       </c>
       <c r="CS69" s="15"/>
     </row>
-    <row r="70" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A70" s="68"/>
       <c r="B70" s="68"/>
       <c r="C70" s="90" t="s">
@@ -18504,7 +18504,7 @@
       </c>
       <c r="CS70" s="82"/>
     </row>
-    <row r="71" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:97" x14ac:dyDescent="0.2">
       <c r="A71" s="68"/>
       <c r="B71" s="68"/>
       <c r="C71" s="89" t="s">
@@ -18657,7 +18657,7 @@
       <c r="CR71" s="51"/>
       <c r="CS71" s="18"/>
     </row>
-    <row r="72" spans="1:97" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:97" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="69"/>
       <c r="B72" s="68"/>
       <c r="C72" s="91" t="s">
@@ -19034,7 +19034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:97" s="97" customFormat="1" ht="16" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:97" s="97" customFormat="1" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="C73" s="98"/>
       <c r="D73" s="46"/>
       <c r="E73" s="46"/>
@@ -19170,7 +19170,7 @@
       </c>
       <c r="CS73" s="101"/>
     </row>
-    <row r="74" spans="1:97" s="97" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:97" s="97" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C74" s="98"/>
       <c r="D74" s="46"/>
       <c r="E74" s="46"/>
@@ -19260,7 +19260,7 @@
       <c r="CK74" s="99"/>
       <c r="CL74" s="99"/>
     </row>
-    <row r="75" spans="1:97" s="84" customFormat="1" ht="20" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:97" s="84" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B75" s="97"/>
       <c r="C75" s="94"/>
       <c r="D75" s="85"/>
@@ -19351,401 +19351,401 @@
       <c r="CK75" s="96"/>
       <c r="CL75" s="96"/>
     </row>
-    <row r="76" spans="1:97" ht="16" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="C76" s="179" t="s">
+    <row r="76" spans="1:97" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="C76" s="181" t="s">
         <v>52</v>
       </c>
       <c r="D76" s="30"/>
       <c r="E76" s="30"/>
       <c r="F76" s="7"/>
-      <c r="G76" s="162">
+      <c r="G76" s="176">
         <f>G$7</f>
         <v>45748</v>
       </c>
-      <c r="H76" s="163"/>
-      <c r="I76" s="163"/>
-      <c r="J76" s="163"/>
-      <c r="K76" s="163"/>
-      <c r="L76" s="163"/>
-      <c r="M76" s="164"/>
-      <c r="N76" s="162">
+      <c r="H76" s="177"/>
+      <c r="I76" s="177"/>
+      <c r="J76" s="177"/>
+      <c r="K76" s="177"/>
+      <c r="L76" s="177"/>
+      <c r="M76" s="178"/>
+      <c r="N76" s="176">
         <f>N$7</f>
         <v>45778</v>
       </c>
-      <c r="O76" s="163"/>
-      <c r="P76" s="163"/>
-      <c r="Q76" s="163"/>
-      <c r="R76" s="163"/>
-      <c r="S76" s="163"/>
-      <c r="T76" s="163"/>
-      <c r="U76" s="162">
+      <c r="O76" s="177"/>
+      <c r="P76" s="177"/>
+      <c r="Q76" s="177"/>
+      <c r="R76" s="177"/>
+      <c r="S76" s="177"/>
+      <c r="T76" s="177"/>
+      <c r="U76" s="176">
         <f>U$7</f>
         <v>45809</v>
       </c>
-      <c r="V76" s="163"/>
-      <c r="W76" s="163"/>
-      <c r="X76" s="163"/>
-      <c r="Y76" s="163"/>
-      <c r="Z76" s="163"/>
-      <c r="AA76" s="164"/>
-      <c r="AB76" s="162">
+      <c r="V76" s="177"/>
+      <c r="W76" s="177"/>
+      <c r="X76" s="177"/>
+      <c r="Y76" s="177"/>
+      <c r="Z76" s="177"/>
+      <c r="AA76" s="178"/>
+      <c r="AB76" s="176">
         <f>AB$7</f>
         <v>45839</v>
       </c>
-      <c r="AC76" s="163"/>
-      <c r="AD76" s="163"/>
-      <c r="AE76" s="163"/>
-      <c r="AF76" s="163"/>
-      <c r="AG76" s="163"/>
-      <c r="AH76" s="164"/>
-      <c r="AI76" s="162">
+      <c r="AC76" s="177"/>
+      <c r="AD76" s="177"/>
+      <c r="AE76" s="177"/>
+      <c r="AF76" s="177"/>
+      <c r="AG76" s="177"/>
+      <c r="AH76" s="178"/>
+      <c r="AI76" s="176">
         <f>AI$7</f>
         <v>45870</v>
       </c>
-      <c r="AJ76" s="163"/>
-      <c r="AK76" s="163"/>
-      <c r="AL76" s="163"/>
-      <c r="AM76" s="163"/>
-      <c r="AN76" s="163"/>
-      <c r="AO76" s="164"/>
-      <c r="AP76" s="162">
+      <c r="AJ76" s="177"/>
+      <c r="AK76" s="177"/>
+      <c r="AL76" s="177"/>
+      <c r="AM76" s="177"/>
+      <c r="AN76" s="177"/>
+      <c r="AO76" s="178"/>
+      <c r="AP76" s="176">
         <f>AP$7</f>
         <v>45901</v>
       </c>
-      <c r="AQ76" s="163"/>
-      <c r="AR76" s="163"/>
-      <c r="AS76" s="163"/>
-      <c r="AT76" s="163"/>
-      <c r="AU76" s="163"/>
-      <c r="AV76" s="164"/>
-      <c r="AW76" s="162">
+      <c r="AQ76" s="177"/>
+      <c r="AR76" s="177"/>
+      <c r="AS76" s="177"/>
+      <c r="AT76" s="177"/>
+      <c r="AU76" s="177"/>
+      <c r="AV76" s="178"/>
+      <c r="AW76" s="176">
         <f>AW$7</f>
         <v>45931</v>
       </c>
-      <c r="AX76" s="163"/>
-      <c r="AY76" s="163"/>
-      <c r="AZ76" s="163"/>
-      <c r="BA76" s="163"/>
-      <c r="BB76" s="163"/>
-      <c r="BC76" s="164"/>
-      <c r="BD76" s="162">
+      <c r="AX76" s="177"/>
+      <c r="AY76" s="177"/>
+      <c r="AZ76" s="177"/>
+      <c r="BA76" s="177"/>
+      <c r="BB76" s="177"/>
+      <c r="BC76" s="178"/>
+      <c r="BD76" s="176">
         <f>BD$7</f>
         <v>45962</v>
       </c>
-      <c r="BE76" s="163"/>
-      <c r="BF76" s="163"/>
-      <c r="BG76" s="163"/>
-      <c r="BH76" s="163"/>
-      <c r="BI76" s="163"/>
-      <c r="BJ76" s="164"/>
-      <c r="BK76" s="162">
+      <c r="BE76" s="177"/>
+      <c r="BF76" s="177"/>
+      <c r="BG76" s="177"/>
+      <c r="BH76" s="177"/>
+      <c r="BI76" s="177"/>
+      <c r="BJ76" s="178"/>
+      <c r="BK76" s="176">
         <f>BK$7</f>
         <v>45992</v>
       </c>
-      <c r="BL76" s="163"/>
-      <c r="BM76" s="163"/>
-      <c r="BN76" s="163"/>
-      <c r="BO76" s="163"/>
-      <c r="BP76" s="163"/>
-      <c r="BQ76" s="164"/>
-      <c r="BR76" s="162">
+      <c r="BL76" s="177"/>
+      <c r="BM76" s="177"/>
+      <c r="BN76" s="177"/>
+      <c r="BO76" s="177"/>
+      <c r="BP76" s="177"/>
+      <c r="BQ76" s="178"/>
+      <c r="BR76" s="176">
         <f>BR$7</f>
         <v>46023</v>
       </c>
-      <c r="BS76" s="163"/>
-      <c r="BT76" s="163"/>
-      <c r="BU76" s="163"/>
-      <c r="BV76" s="163"/>
-      <c r="BW76" s="163"/>
-      <c r="BX76" s="164"/>
-      <c r="BY76" s="162">
+      <c r="BS76" s="177"/>
+      <c r="BT76" s="177"/>
+      <c r="BU76" s="177"/>
+      <c r="BV76" s="177"/>
+      <c r="BW76" s="177"/>
+      <c r="BX76" s="178"/>
+      <c r="BY76" s="176">
         <f>BY$7</f>
         <v>46054</v>
       </c>
-      <c r="BZ76" s="163"/>
-      <c r="CA76" s="163"/>
-      <c r="CB76" s="163"/>
-      <c r="CC76" s="163"/>
-      <c r="CD76" s="163"/>
-      <c r="CE76" s="164"/>
-      <c r="CF76" s="162">
+      <c r="BZ76" s="177"/>
+      <c r="CA76" s="177"/>
+      <c r="CB76" s="177"/>
+      <c r="CC76" s="177"/>
+      <c r="CD76" s="177"/>
+      <c r="CE76" s="178"/>
+      <c r="CF76" s="176">
         <f>CF$7</f>
         <v>46082</v>
       </c>
-      <c r="CG76" s="163"/>
-      <c r="CH76" s="163"/>
-      <c r="CI76" s="163"/>
-      <c r="CJ76" s="163"/>
-      <c r="CK76" s="163"/>
-      <c r="CL76" s="164"/>
-      <c r="CM76" s="162" t="str">
+      <c r="CG76" s="177"/>
+      <c r="CH76" s="177"/>
+      <c r="CI76" s="177"/>
+      <c r="CJ76" s="177"/>
+      <c r="CK76" s="177"/>
+      <c r="CL76" s="178"/>
+      <c r="CM76" s="176" t="str">
         <f>CM$7</f>
         <v>FY26 1H</v>
       </c>
-      <c r="CN76" s="163"/>
-      <c r="CO76" s="163"/>
-      <c r="CP76" s="163"/>
-      <c r="CQ76" s="163"/>
-      <c r="CR76" s="163"/>
-      <c r="CS76" s="164"/>
+      <c r="CN76" s="177"/>
+      <c r="CO76" s="177"/>
+      <c r="CP76" s="177"/>
+      <c r="CQ76" s="177"/>
+      <c r="CR76" s="177"/>
+      <c r="CS76" s="178"/>
     </row>
-    <row r="77" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
-      <c r="C77" s="180"/>
+    <row r="77" spans="1:97" x14ac:dyDescent="0.2">
+      <c r="C77" s="182"/>
       <c r="D77" s="31"/>
       <c r="E77" s="31"/>
       <c r="F77" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G77" s="158" t="str">
+      <c r="G77" s="179" t="str">
         <f>G$8</f>
         <v>Pur</v>
       </c>
-      <c r="H77" s="159"/>
-      <c r="I77" s="160" t="str">
+      <c r="H77" s="175"/>
+      <c r="I77" s="174" t="str">
         <f>I$8</f>
         <v>Consumption</v>
       </c>
-      <c r="J77" s="159"/>
-      <c r="K77" s="160" t="str">
+      <c r="J77" s="175"/>
+      <c r="K77" s="174" t="str">
         <f>K$8</f>
         <v>C/B</v>
       </c>
-      <c r="L77" s="159"/>
+      <c r="L77" s="175"/>
       <c r="M77" s="103" t="str">
         <f>M$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="N77" s="158" t="str">
+      <c r="N77" s="179" t="str">
         <f>N$8</f>
         <v>Pur</v>
       </c>
-      <c r="O77" s="159"/>
-      <c r="P77" s="160" t="str">
+      <c r="O77" s="175"/>
+      <c r="P77" s="174" t="str">
         <f>P$8</f>
         <v>Consumption</v>
       </c>
-      <c r="Q77" s="159"/>
-      <c r="R77" s="160" t="str">
+      <c r="Q77" s="175"/>
+      <c r="R77" s="174" t="str">
         <f>R$8</f>
         <v>C/B</v>
       </c>
-      <c r="S77" s="161"/>
+      <c r="S77" s="180"/>
       <c r="T77" s="104" t="str">
         <f t="shared" ref="T77" si="389">T$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="U77" s="161" t="str">
+      <c r="U77" s="180" t="str">
         <f t="shared" ref="U77" si="390">U$8</f>
         <v>Pur</v>
       </c>
-      <c r="V77" s="159"/>
-      <c r="W77" s="160" t="str">
+      <c r="V77" s="175"/>
+      <c r="W77" s="174" t="str">
         <f t="shared" ref="W77" si="391">W$8</f>
         <v>Consumption</v>
       </c>
-      <c r="X77" s="159"/>
-      <c r="Y77" s="160" t="str">
+      <c r="X77" s="175"/>
+      <c r="Y77" s="174" t="str">
         <f t="shared" ref="Y77" si="392">Y$8</f>
         <v>C/B</v>
       </c>
-      <c r="Z77" s="161"/>
+      <c r="Z77" s="180"/>
       <c r="AA77" s="104" t="str">
         <f t="shared" ref="AA77:AB77" si="393">AA$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AB77" s="158" t="str">
+      <c r="AB77" s="179" t="str">
         <f t="shared" si="393"/>
         <v>Pur</v>
       </c>
-      <c r="AC77" s="159"/>
-      <c r="AD77" s="160" t="str">
+      <c r="AC77" s="175"/>
+      <c r="AD77" s="174" t="str">
         <f t="shared" ref="AD77" si="394">AD$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AE77" s="159"/>
-      <c r="AF77" s="160" t="str">
+      <c r="AE77" s="175"/>
+      <c r="AF77" s="174" t="str">
         <f t="shared" ref="AF77" si="395">AF$8</f>
         <v>C/B</v>
       </c>
-      <c r="AG77" s="161"/>
+      <c r="AG77" s="180"/>
       <c r="AH77" s="104" t="str">
         <f t="shared" ref="AH77:AI77" si="396">AH$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AI77" s="158" t="str">
+      <c r="AI77" s="179" t="str">
         <f t="shared" si="396"/>
         <v>Pur</v>
       </c>
-      <c r="AJ77" s="159"/>
-      <c r="AK77" s="160" t="str">
+      <c r="AJ77" s="175"/>
+      <c r="AK77" s="174" t="str">
         <f t="shared" ref="AK77" si="397">AK$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AL77" s="159"/>
-      <c r="AM77" s="160" t="str">
+      <c r="AL77" s="175"/>
+      <c r="AM77" s="174" t="str">
         <f t="shared" ref="AM77" si="398">AM$8</f>
         <v>C/B</v>
       </c>
-      <c r="AN77" s="161"/>
+      <c r="AN77" s="180"/>
       <c r="AO77" s="105" t="str">
         <f t="shared" ref="AO77:AP77" si="399">AO$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AP77" s="158" t="str">
+      <c r="AP77" s="179" t="str">
         <f t="shared" si="399"/>
         <v>Pur</v>
       </c>
-      <c r="AQ77" s="159"/>
-      <c r="AR77" s="160" t="str">
+      <c r="AQ77" s="175"/>
+      <c r="AR77" s="174" t="str">
         <f t="shared" ref="AR77" si="400">AR$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AS77" s="159"/>
-      <c r="AT77" s="160" t="str">
+      <c r="AS77" s="175"/>
+      <c r="AT77" s="174" t="str">
         <f t="shared" ref="AT77" si="401">AT$8</f>
         <v>C/B</v>
       </c>
-      <c r="AU77" s="161"/>
+      <c r="AU77" s="180"/>
       <c r="AV77" s="104" t="str">
         <f t="shared" ref="AV77:AW77" si="402">AV$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="AW77" s="158" t="str">
+      <c r="AW77" s="179" t="str">
         <f t="shared" si="402"/>
         <v>Pur</v>
       </c>
-      <c r="AX77" s="159"/>
-      <c r="AY77" s="160" t="str">
+      <c r="AX77" s="175"/>
+      <c r="AY77" s="174" t="str">
         <f t="shared" ref="AY77" si="403">AY$8</f>
         <v>Consumption</v>
       </c>
-      <c r="AZ77" s="159"/>
-      <c r="BA77" s="160" t="str">
+      <c r="AZ77" s="175"/>
+      <c r="BA77" s="174" t="str">
         <f t="shared" ref="BA77" si="404">BA$8</f>
         <v>C/B</v>
       </c>
-      <c r="BB77" s="161"/>
+      <c r="BB77" s="180"/>
       <c r="BC77" s="104" t="str">
         <f t="shared" ref="BC77:BD77" si="405">BC$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BD77" s="158" t="str">
+      <c r="BD77" s="179" t="str">
         <f t="shared" si="405"/>
         <v>Pur</v>
       </c>
-      <c r="BE77" s="159"/>
-      <c r="BF77" s="160" t="str">
+      <c r="BE77" s="175"/>
+      <c r="BF77" s="174" t="str">
         <f t="shared" ref="BF77" si="406">BF$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BG77" s="159"/>
-      <c r="BH77" s="160" t="str">
+      <c r="BG77" s="175"/>
+      <c r="BH77" s="174" t="str">
         <f t="shared" ref="BH77" si="407">BH$8</f>
         <v>C/B</v>
       </c>
-      <c r="BI77" s="161"/>
+      <c r="BI77" s="180"/>
       <c r="BJ77" s="104" t="str">
         <f t="shared" ref="BJ77:BK77" si="408">BJ$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BK77" s="158" t="str">
+      <c r="BK77" s="179" t="str">
         <f t="shared" si="408"/>
         <v>Pur</v>
       </c>
-      <c r="BL77" s="159"/>
-      <c r="BM77" s="160" t="str">
+      <c r="BL77" s="175"/>
+      <c r="BM77" s="174" t="str">
         <f t="shared" ref="BM77" si="409">BM$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BN77" s="159"/>
-      <c r="BO77" s="160" t="str">
+      <c r="BN77" s="175"/>
+      <c r="BO77" s="174" t="str">
         <f t="shared" ref="BO77" si="410">BO$8</f>
         <v>C/B</v>
       </c>
-      <c r="BP77" s="161"/>
+      <c r="BP77" s="180"/>
       <c r="BQ77" s="104" t="str">
         <f t="shared" ref="BQ77:BR77" si="411">BQ$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BR77" s="158" t="str">
+      <c r="BR77" s="179" t="str">
         <f t="shared" si="411"/>
         <v>Pur</v>
       </c>
-      <c r="BS77" s="159"/>
-      <c r="BT77" s="160" t="str">
+      <c r="BS77" s="175"/>
+      <c r="BT77" s="174" t="str">
         <f t="shared" ref="BT77" si="412">BT$8</f>
         <v>Consumption</v>
       </c>
-      <c r="BU77" s="159"/>
-      <c r="BV77" s="160" t="str">
+      <c r="BU77" s="175"/>
+      <c r="BV77" s="174" t="str">
         <f t="shared" ref="BV77" si="413">BV$8</f>
         <v>C/B</v>
       </c>
-      <c r="BW77" s="161"/>
+      <c r="BW77" s="180"/>
       <c r="BX77" s="104" t="str">
         <f t="shared" ref="BX77:BY77" si="414">BX$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="BY77" s="158" t="str">
+      <c r="BY77" s="179" t="str">
         <f t="shared" si="414"/>
         <v>Pur</v>
       </c>
-      <c r="BZ77" s="159"/>
-      <c r="CA77" s="160" t="str">
+      <c r="BZ77" s="175"/>
+      <c r="CA77" s="174" t="str">
         <f t="shared" ref="CA77" si="415">CA$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CB77" s="159"/>
-      <c r="CC77" s="160" t="str">
+      <c r="CB77" s="175"/>
+      <c r="CC77" s="174" t="str">
         <f t="shared" ref="CC77" si="416">CC$8</f>
         <v>C/B</v>
       </c>
-      <c r="CD77" s="161"/>
+      <c r="CD77" s="180"/>
       <c r="CE77" s="104" t="str">
         <f t="shared" ref="CE77:CF77" si="417">CE$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="CF77" s="158" t="str">
+      <c r="CF77" s="179" t="str">
         <f t="shared" si="417"/>
         <v>Pur</v>
       </c>
-      <c r="CG77" s="159"/>
-      <c r="CH77" s="160" t="str">
+      <c r="CG77" s="175"/>
+      <c r="CH77" s="174" t="str">
         <f t="shared" ref="CH77" si="418">CH$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CI77" s="159"/>
-      <c r="CJ77" s="160" t="str">
+      <c r="CI77" s="175"/>
+      <c r="CJ77" s="174" t="str">
         <f t="shared" ref="CJ77" si="419">CJ$8</f>
         <v>C/B</v>
       </c>
-      <c r="CK77" s="161"/>
+      <c r="CK77" s="180"/>
       <c r="CL77" s="104" t="str">
         <f t="shared" ref="CL77:CM77" si="420">CL$8</f>
         <v>Inv Days</v>
       </c>
-      <c r="CM77" s="158" t="str">
+      <c r="CM77" s="179" t="str">
         <f t="shared" si="420"/>
         <v>Pur</v>
       </c>
-      <c r="CN77" s="159"/>
-      <c r="CO77" s="160" t="str">
+      <c r="CN77" s="175"/>
+      <c r="CO77" s="174" t="str">
         <f t="shared" ref="CO77" si="421">CO$8</f>
         <v>Consumption</v>
       </c>
-      <c r="CP77" s="159"/>
-      <c r="CQ77" s="160" t="str">
+      <c r="CP77" s="175"/>
+      <c r="CQ77" s="174" t="str">
         <f t="shared" ref="CQ77" si="422">CQ$8</f>
         <v>C/B</v>
       </c>
-      <c r="CR77" s="161"/>
+      <c r="CR77" s="180"/>
       <c r="CS77" s="104" t="str">
         <f t="shared" ref="CS77" si="423">CS$8</f>
         <v>Inv Days</v>
       </c>
     </row>
-    <row r="78" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
-      <c r="C78" s="181"/>
+    <row r="78" spans="1:97" x14ac:dyDescent="0.2">
+      <c r="C78" s="183"/>
       <c r="D78" s="32"/>
       <c r="E78" s="32"/>
       <c r="F78" s="8" t="str">
@@ -20117,7 +20117,7 @@
         <v>T/F</v>
       </c>
     </row>
-    <row r="79" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:97" x14ac:dyDescent="0.2">
       <c r="C79" s="93" t="s">
         <v>53</v>
       </c>
@@ -20492,7 +20492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:97" x14ac:dyDescent="0.2">
       <c r="C80" s="93" t="s">
         <v>54</v>
       </c>
@@ -20867,7 +20867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="3:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="3:97" x14ac:dyDescent="0.2">
       <c r="C81" s="93" t="s">
         <v>55</v>
       </c>
@@ -21242,7 +21242,7 @@
         <v>329.78440334860863</v>
       </c>
     </row>
-    <row r="82" spans="3:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="3:97" x14ac:dyDescent="0.2">
       <c r="C82" s="93" t="s">
         <v>56</v>
       </c>
@@ -21617,7 +21617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="3:97" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:97" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C83" s="91" t="s">
         <v>57</v>
       </c>
@@ -21992,7 +21992,7 @@
         <v>39.648893275351462</v>
       </c>
     </row>
-    <row r="84" spans="3:97" s="69" customFormat="1" ht="16" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="3:97" s="69" customFormat="1" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="C84" s="126"/>
       <c r="D84" s="127"/>
       <c r="E84" s="127"/>
@@ -22052,7 +22052,7 @@
       </c>
       <c r="CL84" s="128"/>
     </row>
-    <row r="85" spans="3:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="3:97" x14ac:dyDescent="0.2">
       <c r="F85" s="57"/>
       <c r="L85" s="57"/>
       <c r="Z85" s="45"/>
@@ -22067,7 +22067,7 @@
       <c r="CJ85" s="54"/>
       <c r="CK85" s="54"/>
     </row>
-    <row r="86" spans="3:97" s="69" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="3:97" s="69" customFormat="1" x14ac:dyDescent="0.2">
       <c r="C86" s="126"/>
       <c r="D86" s="127"/>
       <c r="E86" s="127"/>
@@ -22150,7 +22150,7 @@
       </c>
       <c r="CL86" s="128"/>
     </row>
-    <row r="87" spans="3:97" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="3:97" x14ac:dyDescent="0.2">
       <c r="L87" s="73"/>
       <c r="AU87" s="95"/>
     </row>
@@ -22300,7 +22300,7 @@
         <v>4886.8312757201647</v>
       </c>
       <c r="S93" s="57">
-        <f t="shared" ref="S92:S102" si="497">Q93-R93</f>
+        <f t="shared" ref="S93:S102" si="497">Q93-R93</f>
         <v>2545.222790928924</v>
       </c>
     </row>
@@ -22638,6 +22638,259 @@
     </row>
   </sheetData>
   <mergeCells count="277">
+    <mergeCell ref="CM77:CN77"/>
+    <mergeCell ref="CO77:CP77"/>
+    <mergeCell ref="CQ77:CR77"/>
+    <mergeCell ref="CM76:CS76"/>
+    <mergeCell ref="CM59:CS59"/>
+    <mergeCell ref="CM60:CN60"/>
+    <mergeCell ref="CO60:CP60"/>
+    <mergeCell ref="CQ60:CR60"/>
+    <mergeCell ref="CM40:CS40"/>
+    <mergeCell ref="CM41:CN41"/>
+    <mergeCell ref="CO41:CP41"/>
+    <mergeCell ref="CQ41:CR41"/>
+    <mergeCell ref="CM24:CN24"/>
+    <mergeCell ref="CO24:CP24"/>
+    <mergeCell ref="CQ24:CR24"/>
+    <mergeCell ref="CM7:CS7"/>
+    <mergeCell ref="CM8:CN8"/>
+    <mergeCell ref="CO8:CP8"/>
+    <mergeCell ref="CQ8:CR8"/>
+    <mergeCell ref="CF7:CL7"/>
+    <mergeCell ref="BR23:BX23"/>
+    <mergeCell ref="BY23:CE23"/>
+    <mergeCell ref="CF23:CL23"/>
+    <mergeCell ref="CJ8:CK8"/>
+    <mergeCell ref="CM23:CS23"/>
+    <mergeCell ref="CH24:CI24"/>
+    <mergeCell ref="CJ24:CK24"/>
+    <mergeCell ref="BR24:BS24"/>
+    <mergeCell ref="BT24:BU24"/>
+    <mergeCell ref="BV24:BW24"/>
+    <mergeCell ref="BK7:BQ7"/>
+    <mergeCell ref="BR7:BX7"/>
+    <mergeCell ref="BY7:CE7"/>
+    <mergeCell ref="CA8:CB8"/>
+    <mergeCell ref="CH8:CI8"/>
+    <mergeCell ref="BR8:BS8"/>
+    <mergeCell ref="BT8:BU8"/>
+    <mergeCell ref="BV8:BW8"/>
+    <mergeCell ref="BY8:BZ8"/>
+    <mergeCell ref="BK23:BQ23"/>
+    <mergeCell ref="BK8:BL8"/>
+    <mergeCell ref="BM8:BN8"/>
+    <mergeCell ref="BO8:BP8"/>
+    <mergeCell ref="CC8:CD8"/>
+    <mergeCell ref="CF8:CG8"/>
+    <mergeCell ref="CA24:CB24"/>
+    <mergeCell ref="CC24:CD24"/>
+    <mergeCell ref="AK41:AL41"/>
+    <mergeCell ref="CF24:CG24"/>
+    <mergeCell ref="AM41:AN41"/>
+    <mergeCell ref="BK41:BL41"/>
+    <mergeCell ref="BD8:BE8"/>
+    <mergeCell ref="AP23:AV23"/>
+    <mergeCell ref="BD41:BE41"/>
+    <mergeCell ref="BF41:BG41"/>
+    <mergeCell ref="AW23:BC23"/>
+    <mergeCell ref="BD23:BJ23"/>
+    <mergeCell ref="BM41:BN41"/>
+    <mergeCell ref="BO41:BP41"/>
+    <mergeCell ref="AK8:AL8"/>
+    <mergeCell ref="CF40:CL40"/>
+    <mergeCell ref="AM24:AN24"/>
+    <mergeCell ref="AP24:AQ24"/>
+    <mergeCell ref="BY40:CE40"/>
+    <mergeCell ref="AW24:AX24"/>
+    <mergeCell ref="BY24:BZ24"/>
+    <mergeCell ref="BR40:BX40"/>
+    <mergeCell ref="BK24:BL24"/>
+    <mergeCell ref="AI40:AO40"/>
+    <mergeCell ref="AK24:AL24"/>
+    <mergeCell ref="AT24:AU24"/>
+    <mergeCell ref="AR24:AS24"/>
+    <mergeCell ref="AP40:AV40"/>
+    <mergeCell ref="BK40:BQ40"/>
+    <mergeCell ref="BO24:BP24"/>
+    <mergeCell ref="BM24:BN24"/>
+    <mergeCell ref="AW7:BC7"/>
+    <mergeCell ref="BD7:BJ7"/>
+    <mergeCell ref="AP8:AQ8"/>
+    <mergeCell ref="AR8:AS8"/>
+    <mergeCell ref="AT8:AU8"/>
+    <mergeCell ref="BH41:BI41"/>
+    <mergeCell ref="AW40:BC40"/>
+    <mergeCell ref="AW8:AX8"/>
+    <mergeCell ref="AY8:AZ8"/>
+    <mergeCell ref="BA8:BB8"/>
+    <mergeCell ref="BH8:BI8"/>
+    <mergeCell ref="BF8:BG8"/>
+    <mergeCell ref="BD40:BJ40"/>
+    <mergeCell ref="AY24:AZ24"/>
+    <mergeCell ref="BA24:BB24"/>
+    <mergeCell ref="BD24:BE24"/>
+    <mergeCell ref="BF24:BG24"/>
+    <mergeCell ref="BH24:BI24"/>
+    <mergeCell ref="AP7:AV7"/>
+    <mergeCell ref="U60:V60"/>
+    <mergeCell ref="AK60:AL60"/>
+    <mergeCell ref="AM60:AN60"/>
+    <mergeCell ref="W60:X60"/>
+    <mergeCell ref="Y60:Z60"/>
+    <mergeCell ref="AI60:AJ60"/>
+    <mergeCell ref="AP60:AQ60"/>
+    <mergeCell ref="AI59:AO59"/>
+    <mergeCell ref="AY41:AZ41"/>
+    <mergeCell ref="AW59:BC59"/>
+    <mergeCell ref="AR41:AS41"/>
+    <mergeCell ref="AT41:AU41"/>
+    <mergeCell ref="AW41:AX41"/>
+    <mergeCell ref="AB59:AH59"/>
+    <mergeCell ref="AB60:AC60"/>
+    <mergeCell ref="AD60:AE60"/>
+    <mergeCell ref="AF60:AG60"/>
+    <mergeCell ref="AP59:AV59"/>
+    <mergeCell ref="AR60:AS60"/>
+    <mergeCell ref="AT60:AU60"/>
+    <mergeCell ref="AP41:AQ41"/>
+    <mergeCell ref="U59:AA59"/>
+    <mergeCell ref="AI41:AJ41"/>
+    <mergeCell ref="AW60:AX60"/>
+    <mergeCell ref="BK60:BL60"/>
+    <mergeCell ref="BM60:BN60"/>
+    <mergeCell ref="BO60:BP60"/>
+    <mergeCell ref="BY59:CE59"/>
+    <mergeCell ref="BK59:BQ59"/>
+    <mergeCell ref="BA41:BB41"/>
+    <mergeCell ref="BH60:BI60"/>
+    <mergeCell ref="BD60:BE60"/>
+    <mergeCell ref="AY60:AZ60"/>
+    <mergeCell ref="BA60:BB60"/>
+    <mergeCell ref="BF60:BG60"/>
+    <mergeCell ref="BD59:BJ59"/>
+    <mergeCell ref="CF59:CL59"/>
+    <mergeCell ref="BR41:BS41"/>
+    <mergeCell ref="BT41:BU41"/>
+    <mergeCell ref="BV41:BW41"/>
+    <mergeCell ref="BY41:BZ41"/>
+    <mergeCell ref="CA41:CB41"/>
+    <mergeCell ref="CC41:CD41"/>
+    <mergeCell ref="CF60:CG60"/>
+    <mergeCell ref="CH60:CI60"/>
+    <mergeCell ref="BR60:BS60"/>
+    <mergeCell ref="BT60:BU60"/>
+    <mergeCell ref="BV60:BW60"/>
+    <mergeCell ref="BY60:BZ60"/>
+    <mergeCell ref="CA60:CB60"/>
+    <mergeCell ref="CF41:CG41"/>
+    <mergeCell ref="CH41:CI41"/>
+    <mergeCell ref="CJ41:CK41"/>
+    <mergeCell ref="CC60:CD60"/>
+    <mergeCell ref="CJ60:CK60"/>
+    <mergeCell ref="BR59:BX59"/>
+    <mergeCell ref="CF76:CL76"/>
+    <mergeCell ref="BR76:BX76"/>
+    <mergeCell ref="BY76:CE76"/>
+    <mergeCell ref="BO77:BP77"/>
+    <mergeCell ref="AP77:AQ77"/>
+    <mergeCell ref="AR77:AS77"/>
+    <mergeCell ref="AT77:AU77"/>
+    <mergeCell ref="AW77:AX77"/>
+    <mergeCell ref="AY77:AZ77"/>
+    <mergeCell ref="BA77:BB77"/>
+    <mergeCell ref="BD77:BE77"/>
+    <mergeCell ref="BF77:BG77"/>
+    <mergeCell ref="BR77:BS77"/>
+    <mergeCell ref="BT77:BU77"/>
+    <mergeCell ref="BV77:BW77"/>
+    <mergeCell ref="BY77:BZ77"/>
+    <mergeCell ref="CA77:CB77"/>
+    <mergeCell ref="BM77:BN77"/>
+    <mergeCell ref="BK76:BQ76"/>
+    <mergeCell ref="BK77:BL77"/>
+    <mergeCell ref="CC77:CD77"/>
+    <mergeCell ref="CF77:CG77"/>
+    <mergeCell ref="CH77:CI77"/>
+    <mergeCell ref="CJ77:CK77"/>
+    <mergeCell ref="AM77:AN77"/>
+    <mergeCell ref="U77:V77"/>
+    <mergeCell ref="W77:X77"/>
+    <mergeCell ref="AI76:AO76"/>
+    <mergeCell ref="AP76:AV76"/>
+    <mergeCell ref="AW76:BC76"/>
+    <mergeCell ref="BD76:BJ76"/>
+    <mergeCell ref="Y77:Z77"/>
+    <mergeCell ref="AB77:AC77"/>
+    <mergeCell ref="U76:AA76"/>
+    <mergeCell ref="BH77:BI77"/>
+    <mergeCell ref="AB76:AH76"/>
+    <mergeCell ref="AD77:AE77"/>
+    <mergeCell ref="AF77:AG77"/>
+    <mergeCell ref="AI77:AJ77"/>
+    <mergeCell ref="AK77:AL77"/>
+    <mergeCell ref="K77:L77"/>
+    <mergeCell ref="C59:C61"/>
+    <mergeCell ref="G60:H60"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="K60:L60"/>
+    <mergeCell ref="N60:O60"/>
+    <mergeCell ref="G76:M76"/>
+    <mergeCell ref="G59:M59"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="E60:E61"/>
+    <mergeCell ref="N77:O77"/>
+    <mergeCell ref="N59:T59"/>
+    <mergeCell ref="P77:Q77"/>
+    <mergeCell ref="P60:Q60"/>
+    <mergeCell ref="R77:S77"/>
+    <mergeCell ref="N76:T76"/>
+    <mergeCell ref="C76:C78"/>
+    <mergeCell ref="G77:H77"/>
+    <mergeCell ref="I77:J77"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="R60:S60"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="G40:M40"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="AB24:AC24"/>
+    <mergeCell ref="AF24:AG24"/>
+    <mergeCell ref="AF8:AG8"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="W8:X8"/>
+    <mergeCell ref="Y8:Z8"/>
+    <mergeCell ref="AI24:AJ24"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="G7:M7"/>
+    <mergeCell ref="G23:M23"/>
+    <mergeCell ref="AI8:AJ8"/>
+    <mergeCell ref="N7:T7"/>
+    <mergeCell ref="N23:T23"/>
+    <mergeCell ref="AI7:AO7"/>
+    <mergeCell ref="AI23:AO23"/>
+    <mergeCell ref="AB7:AH7"/>
+    <mergeCell ref="U7:AA7"/>
+    <mergeCell ref="AM8:AN8"/>
+    <mergeCell ref="U23:AA23"/>
     <mergeCell ref="N41:O41"/>
     <mergeCell ref="P41:Q41"/>
     <mergeCell ref="R41:S41"/>
@@ -22662,259 +22915,6 @@
     <mergeCell ref="Y24:Z24"/>
     <mergeCell ref="P8:Q8"/>
     <mergeCell ref="R8:S8"/>
-    <mergeCell ref="AB24:AC24"/>
-    <mergeCell ref="AF24:AG24"/>
-    <mergeCell ref="AF8:AG8"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U8:V8"/>
-    <mergeCell ref="W8:X8"/>
-    <mergeCell ref="Y8:Z8"/>
-    <mergeCell ref="AI24:AJ24"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="G7:M7"/>
-    <mergeCell ref="G23:M23"/>
-    <mergeCell ref="AI8:AJ8"/>
-    <mergeCell ref="N7:T7"/>
-    <mergeCell ref="N23:T23"/>
-    <mergeCell ref="AI7:AO7"/>
-    <mergeCell ref="AI23:AO23"/>
-    <mergeCell ref="AB7:AH7"/>
-    <mergeCell ref="U7:AA7"/>
-    <mergeCell ref="AM8:AN8"/>
-    <mergeCell ref="U23:AA23"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="G40:M40"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="C40:C42"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="K41:L41"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="K77:L77"/>
-    <mergeCell ref="C59:C61"/>
-    <mergeCell ref="G60:H60"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="K60:L60"/>
-    <mergeCell ref="N60:O60"/>
-    <mergeCell ref="G76:M76"/>
-    <mergeCell ref="G59:M59"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="E60:E61"/>
-    <mergeCell ref="N77:O77"/>
-    <mergeCell ref="N59:T59"/>
-    <mergeCell ref="P77:Q77"/>
-    <mergeCell ref="P60:Q60"/>
-    <mergeCell ref="R77:S77"/>
-    <mergeCell ref="N76:T76"/>
-    <mergeCell ref="C76:C78"/>
-    <mergeCell ref="G77:H77"/>
-    <mergeCell ref="I77:J77"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="R60:S60"/>
-    <mergeCell ref="AM77:AN77"/>
-    <mergeCell ref="U77:V77"/>
-    <mergeCell ref="W77:X77"/>
-    <mergeCell ref="AI76:AO76"/>
-    <mergeCell ref="AP76:AV76"/>
-    <mergeCell ref="AW76:BC76"/>
-    <mergeCell ref="BD76:BJ76"/>
-    <mergeCell ref="Y77:Z77"/>
-    <mergeCell ref="AB77:AC77"/>
-    <mergeCell ref="U76:AA76"/>
-    <mergeCell ref="BH77:BI77"/>
-    <mergeCell ref="AB76:AH76"/>
-    <mergeCell ref="AD77:AE77"/>
-    <mergeCell ref="AF77:AG77"/>
-    <mergeCell ref="AI77:AJ77"/>
-    <mergeCell ref="AK77:AL77"/>
-    <mergeCell ref="CF76:CL76"/>
-    <mergeCell ref="BR76:BX76"/>
-    <mergeCell ref="BY76:CE76"/>
-    <mergeCell ref="BO77:BP77"/>
-    <mergeCell ref="AP77:AQ77"/>
-    <mergeCell ref="AR77:AS77"/>
-    <mergeCell ref="AT77:AU77"/>
-    <mergeCell ref="AW77:AX77"/>
-    <mergeCell ref="AY77:AZ77"/>
-    <mergeCell ref="BA77:BB77"/>
-    <mergeCell ref="BD77:BE77"/>
-    <mergeCell ref="BF77:BG77"/>
-    <mergeCell ref="BR77:BS77"/>
-    <mergeCell ref="BT77:BU77"/>
-    <mergeCell ref="BV77:BW77"/>
-    <mergeCell ref="BY77:BZ77"/>
-    <mergeCell ref="CA77:CB77"/>
-    <mergeCell ref="BM77:BN77"/>
-    <mergeCell ref="BK76:BQ76"/>
-    <mergeCell ref="BK77:BL77"/>
-    <mergeCell ref="CC77:CD77"/>
-    <mergeCell ref="CF77:CG77"/>
-    <mergeCell ref="CH77:CI77"/>
-    <mergeCell ref="CJ77:CK77"/>
-    <mergeCell ref="CF59:CL59"/>
-    <mergeCell ref="BR41:BS41"/>
-    <mergeCell ref="BT41:BU41"/>
-    <mergeCell ref="BV41:BW41"/>
-    <mergeCell ref="BY41:BZ41"/>
-    <mergeCell ref="CA41:CB41"/>
-    <mergeCell ref="CC41:CD41"/>
-    <mergeCell ref="CF60:CG60"/>
-    <mergeCell ref="CH60:CI60"/>
-    <mergeCell ref="BR60:BS60"/>
-    <mergeCell ref="BT60:BU60"/>
-    <mergeCell ref="BV60:BW60"/>
-    <mergeCell ref="BY60:BZ60"/>
-    <mergeCell ref="CA60:CB60"/>
-    <mergeCell ref="CF41:CG41"/>
-    <mergeCell ref="CH41:CI41"/>
-    <mergeCell ref="CJ41:CK41"/>
-    <mergeCell ref="CC60:CD60"/>
-    <mergeCell ref="CJ60:CK60"/>
-    <mergeCell ref="BR59:BX59"/>
-    <mergeCell ref="BK60:BL60"/>
-    <mergeCell ref="BM60:BN60"/>
-    <mergeCell ref="BO60:BP60"/>
-    <mergeCell ref="BY59:CE59"/>
-    <mergeCell ref="BK59:BQ59"/>
-    <mergeCell ref="BA41:BB41"/>
-    <mergeCell ref="BH60:BI60"/>
-    <mergeCell ref="BD60:BE60"/>
-    <mergeCell ref="AY60:AZ60"/>
-    <mergeCell ref="BA60:BB60"/>
-    <mergeCell ref="BF60:BG60"/>
-    <mergeCell ref="BD59:BJ59"/>
-    <mergeCell ref="U60:V60"/>
-    <mergeCell ref="AK60:AL60"/>
-    <mergeCell ref="AM60:AN60"/>
-    <mergeCell ref="W60:X60"/>
-    <mergeCell ref="Y60:Z60"/>
-    <mergeCell ref="AI60:AJ60"/>
-    <mergeCell ref="AP60:AQ60"/>
-    <mergeCell ref="AI59:AO59"/>
-    <mergeCell ref="AY41:AZ41"/>
-    <mergeCell ref="AW59:BC59"/>
-    <mergeCell ref="AR41:AS41"/>
-    <mergeCell ref="AT41:AU41"/>
-    <mergeCell ref="AW41:AX41"/>
-    <mergeCell ref="AB59:AH59"/>
-    <mergeCell ref="AB60:AC60"/>
-    <mergeCell ref="AD60:AE60"/>
-    <mergeCell ref="AF60:AG60"/>
-    <mergeCell ref="AP59:AV59"/>
-    <mergeCell ref="AR60:AS60"/>
-    <mergeCell ref="AT60:AU60"/>
-    <mergeCell ref="AP41:AQ41"/>
-    <mergeCell ref="U59:AA59"/>
-    <mergeCell ref="AI41:AJ41"/>
-    <mergeCell ref="AW60:AX60"/>
-    <mergeCell ref="AW7:BC7"/>
-    <mergeCell ref="BD7:BJ7"/>
-    <mergeCell ref="AP8:AQ8"/>
-    <mergeCell ref="AR8:AS8"/>
-    <mergeCell ref="AT8:AU8"/>
-    <mergeCell ref="BH41:BI41"/>
-    <mergeCell ref="AW40:BC40"/>
-    <mergeCell ref="AW8:AX8"/>
-    <mergeCell ref="AY8:AZ8"/>
-    <mergeCell ref="BA8:BB8"/>
-    <mergeCell ref="BH8:BI8"/>
-    <mergeCell ref="BF8:BG8"/>
-    <mergeCell ref="BD40:BJ40"/>
-    <mergeCell ref="AY24:AZ24"/>
-    <mergeCell ref="BA24:BB24"/>
-    <mergeCell ref="BD24:BE24"/>
-    <mergeCell ref="BF24:BG24"/>
-    <mergeCell ref="BH24:BI24"/>
-    <mergeCell ref="AP7:AV7"/>
-    <mergeCell ref="BY40:CE40"/>
-    <mergeCell ref="AW24:AX24"/>
-    <mergeCell ref="BY24:BZ24"/>
-    <mergeCell ref="BR40:BX40"/>
-    <mergeCell ref="BK24:BL24"/>
-    <mergeCell ref="AI40:AO40"/>
-    <mergeCell ref="AK24:AL24"/>
-    <mergeCell ref="AT24:AU24"/>
-    <mergeCell ref="AR24:AS24"/>
-    <mergeCell ref="AP40:AV40"/>
-    <mergeCell ref="BK40:BQ40"/>
-    <mergeCell ref="BO24:BP24"/>
-    <mergeCell ref="BM24:BN24"/>
-    <mergeCell ref="BK23:BQ23"/>
-    <mergeCell ref="BK8:BL8"/>
-    <mergeCell ref="BM8:BN8"/>
-    <mergeCell ref="BO8:BP8"/>
-    <mergeCell ref="CC8:CD8"/>
-    <mergeCell ref="CF8:CG8"/>
-    <mergeCell ref="CA24:CB24"/>
-    <mergeCell ref="CC24:CD24"/>
-    <mergeCell ref="AK41:AL41"/>
-    <mergeCell ref="CF24:CG24"/>
-    <mergeCell ref="AM41:AN41"/>
-    <mergeCell ref="BK41:BL41"/>
-    <mergeCell ref="BD8:BE8"/>
-    <mergeCell ref="AP23:AV23"/>
-    <mergeCell ref="BD41:BE41"/>
-    <mergeCell ref="BF41:BG41"/>
-    <mergeCell ref="AW23:BC23"/>
-    <mergeCell ref="BD23:BJ23"/>
-    <mergeCell ref="BM41:BN41"/>
-    <mergeCell ref="BO41:BP41"/>
-    <mergeCell ref="AK8:AL8"/>
-    <mergeCell ref="CF40:CL40"/>
-    <mergeCell ref="AM24:AN24"/>
-    <mergeCell ref="AP24:AQ24"/>
-    <mergeCell ref="BK7:BQ7"/>
-    <mergeCell ref="BR7:BX7"/>
-    <mergeCell ref="BY7:CE7"/>
-    <mergeCell ref="CA8:CB8"/>
-    <mergeCell ref="CH8:CI8"/>
-    <mergeCell ref="BR8:BS8"/>
-    <mergeCell ref="BT8:BU8"/>
-    <mergeCell ref="BV8:BW8"/>
-    <mergeCell ref="BY8:BZ8"/>
-    <mergeCell ref="CM24:CN24"/>
-    <mergeCell ref="CO24:CP24"/>
-    <mergeCell ref="CQ24:CR24"/>
-    <mergeCell ref="CM7:CS7"/>
-    <mergeCell ref="CM8:CN8"/>
-    <mergeCell ref="CO8:CP8"/>
-    <mergeCell ref="CQ8:CR8"/>
-    <mergeCell ref="CF7:CL7"/>
-    <mergeCell ref="BR23:BX23"/>
-    <mergeCell ref="BY23:CE23"/>
-    <mergeCell ref="CF23:CL23"/>
-    <mergeCell ref="CJ8:CK8"/>
-    <mergeCell ref="CM23:CS23"/>
-    <mergeCell ref="CH24:CI24"/>
-    <mergeCell ref="CJ24:CK24"/>
-    <mergeCell ref="BR24:BS24"/>
-    <mergeCell ref="BT24:BU24"/>
-    <mergeCell ref="BV24:BW24"/>
-    <mergeCell ref="CM77:CN77"/>
-    <mergeCell ref="CO77:CP77"/>
-    <mergeCell ref="CQ77:CR77"/>
-    <mergeCell ref="CM76:CS76"/>
-    <mergeCell ref="CM59:CS59"/>
-    <mergeCell ref="CM60:CN60"/>
-    <mergeCell ref="CO60:CP60"/>
-    <mergeCell ref="CQ60:CR60"/>
-    <mergeCell ref="CM40:CS40"/>
-    <mergeCell ref="CM41:CN41"/>
-    <mergeCell ref="CO41:CP41"/>
-    <mergeCell ref="CQ41:CR41"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="A19:XFD19 CM20 A36:W36 Y36:AR36 AT36:XFD36 A55:XFD55 A73:XFD73">

</xml_diff>